<commit_message>
Add 44 sourced products to the gear catalog and link 20 cost guide rows
Covers the 40 top-priority lines in NEEDS_PRODUCT.md (seasonal, wide reach
and repeat purchase). Amazon dp links tagged beastlyfacts-20; price, rating
and image wait for a check on the live listing. Crested gecko's cost guide
gains its first affiliate link, so it now carries the disclosure. Finished
lines move to archive/docs-completed/NEEDS_PRODUCT_COMPLETED_2026-09-28.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012EvHa8anGf58M3dpjKW87b
</commit_message>
<xml_diff>
--- a/NEEDS_PRODUCT.xlsx
+++ b/NEEDS_PRODUCT.xlsx
@@ -1205,12 +1205,12 @@
       </c>
       <c r="I15" s="29" t="inlineStr">
         <is>
-          <t>Link found</t>
+          <t>Added to catalog</t>
         </is>
       </c>
       <c r="J15" s="28" t="inlineStr">
         <is>
-          <t>Inkbird IHC200 plug-in humidistat</t>
+          <t>Inkbird IHC200 Plug-In Humidity Controller (Humidistat)</t>
         </is>
       </c>
       <c r="K15" s="29" t="inlineStr">
@@ -1238,11 +1238,19 @@
         </is>
       </c>
       <c r="P15" s="31" t="n"/>
-      <c r="Q15" s="29" t="n"/>
-      <c r="R15" s="32" t="n"/>
+      <c r="Q15" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R15" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="S15" s="28" t="inlineStr">
         <is>
-          <t>Sourced 2026-09-28 from Amazon search results; price not visible from here. Two parts. Humidifier: Everlasting Comfort 6L Cool Mist (B077Z2QCS5); alt Levoit 6L (B08HS45N13). The humidistat only cuts power, so the humidifier must resume misting when power returns (knob models do, touch-button models like Levoit often do not). Check the Everlasting Comfort controls before publishing.</t>
+          <t>Catalog slug: humidistat-inkbird-ihc200, humidifier-everlasting-comfort-6l. Also added: Everlasting Comfort 6L Cool Mist Ultrasonic Humidifier (https://www.amazon.com/dp/B077Z2QCS5). Sourced 2026-09-28 from Amazon search results; price not visible from here. Two parts. Humidifier: Everlasting Comfort 6L Cool Mist (B077Z2QCS5); alt Levoit 6L (B08HS45N13). The humidistat only cuts power, so the humidifier must resume misting when power returns (knob models do, touch-button models like Levoit often do not). Check the Everlasting Comfort controls before publishing.</t>
         </is>
       </c>
     </row>
@@ -1283,12 +1291,12 @@
       <c r="H16" s="28" t="inlineStr"/>
       <c r="I16" s="29" t="inlineStr">
         <is>
-          <t>Link found</t>
+          <t>Added to catalog</t>
         </is>
       </c>
       <c r="J16" s="28" t="inlineStr">
         <is>
-          <t>Zoo Med Reptile Basking Spot Lamp 25W</t>
+          <t>Zoo Med Reptile Basking Spot Lamp, 25W</t>
         </is>
       </c>
       <c r="K16" s="29" t="inlineStr">
@@ -1316,11 +1324,19 @@
         </is>
       </c>
       <c r="P16" s="31" t="n"/>
-      <c r="Q16" s="29" t="n"/>
-      <c r="R16" s="32" t="n"/>
+      <c r="Q16" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R16" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="S16" s="28" t="inlineStr">
         <is>
-          <t>Sourced 2026-09-28 from Amazon search results; price not visible from here. No 40W Zoo Med or Exo Terra basking bulb found on Amazon. Alt: Zoo Med Daylight Blue 25W (B0002AQD1S).</t>
+          <t>Catalog slug: heat-bulb-zoo-med-basking-spot-25w. Sourced 2026-09-28 from Amazon search results; price not visible from here. No 40W Zoo Med or Exo Terra basking bulb found on Amazon. Alt: Zoo Med Daylight Blue 25W (B0002AQD1S).</t>
         </is>
       </c>
     </row>
@@ -1361,12 +1377,12 @@
       <c r="H17" s="28" t="inlineStr"/>
       <c r="I17" s="29" t="inlineStr">
         <is>
-          <t>Link found</t>
+          <t>Added to catalog</t>
         </is>
       </c>
       <c r="J17" s="28" t="inlineStr">
         <is>
-          <t>Arcadia Deep Heat Projector 80W</t>
+          <t>Arcadia Deep Heat Projector, 80W</t>
         </is>
       </c>
       <c r="K17" s="29" t="inlineStr">
@@ -1394,11 +1410,19 @@
         </is>
       </c>
       <c r="P17" s="31" t="n"/>
-      <c r="Q17" s="29" t="n"/>
-      <c r="R17" s="32" t="n"/>
+      <c r="Q17" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R17" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="S17" s="28" t="inlineStr">
         <is>
-          <t>Sourced 2026-09-28 from Amazon search results; price not visible from here. Alt: Arcadia Deep Heat Emitter 50W (B0BSHS996Y).</t>
+          <t>Catalog slug: deep-heat-projector-arcadia-80w. Sourced 2026-09-28 from Amazon search results; price not visible from here. Alt: Arcadia Deep Heat Emitter 50W (B0BSHS996Y).</t>
         </is>
       </c>
     </row>
@@ -1439,7 +1463,7 @@
       <c r="H18" s="28" t="inlineStr"/>
       <c r="I18" s="29" t="inlineStr">
         <is>
-          <t>Link found</t>
+          <t>Added to catalog</t>
         </is>
       </c>
       <c r="J18" s="28" t="inlineStr">
@@ -1472,11 +1496,19 @@
         </is>
       </c>
       <c r="P18" s="31" t="n"/>
-      <c r="Q18" s="29" t="n"/>
-      <c r="R18" s="32" t="n"/>
+      <c r="Q18" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R18" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="S18" s="28" t="inlineStr">
         <is>
-          <t>Sourced 2026-09-28 from Amazon search results; price not visible from here. True overhead RHP. Alt: WARHP Wilbanks 220W (B0HGHMBPTD). Avoid B01N7G3CPP (28W bundled with disinfectant).</t>
+          <t>Catalog slug: radiant-heat-panel-reptile-basics-80w. Sourced 2026-09-28 from Amazon search results; price not visible from here. True overhead RHP. Alt: WARHP Wilbanks 220W (B0HGHMBPTD). Avoid B01N7G3CPP (28W bundled with disinfectant).</t>
         </is>
       </c>
     </row>
@@ -1521,12 +1553,12 @@
       </c>
       <c r="I19" s="29" t="inlineStr">
         <is>
-          <t>Link found</t>
+          <t>Added to catalog</t>
         </is>
       </c>
       <c r="J19" s="28" t="inlineStr">
         <is>
-          <t>Vinaco PAR30 Long Neck 75W Halogen Flood, 6 Pack</t>
+          <t>Vinaco PAR30 Long Neck 75W Halogen Flood Bulbs, 6 Pack</t>
         </is>
       </c>
       <c r="K19" s="29" t="inlineStr">
@@ -1554,11 +1586,19 @@
         </is>
       </c>
       <c r="P19" s="31" t="n"/>
-      <c r="Q19" s="29" t="n"/>
-      <c r="R19" s="32" t="n"/>
+      <c r="Q19" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R19" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="S19" s="28" t="inlineStr">
         <is>
-          <t>Sourced 2026-09-28 from Amazon search results; price not visible from here. Picked over Philips 419549 6-pack (B01MDM2PSL) because the Philips title says "75 Watt Equivalent", which may mean a lower real draw. Catalog already has Zoo Med Basking Spot Lamp 75W 2-pack (not halogen, unwired).</t>
+          <t>Catalog slug: halogen-flood-vinaco-par30-75w-6pack. Sourced 2026-09-28 from Amazon search results; price not visible from here. Picked over Philips 419549 6-pack (B01MDM2PSL) because the Philips title says "75 Watt Equivalent", which may mean a lower real draw. Catalog already has Zoo Med Basking Spot Lamp 75W 2-pack (not halogen, unwired).</t>
         </is>
       </c>
     </row>
@@ -1599,12 +1639,12 @@
       <c r="H20" s="28" t="inlineStr"/>
       <c r="I20" s="29" t="inlineStr">
         <is>
-          <t>Link found</t>
+          <t>Added to catalog</t>
         </is>
       </c>
       <c r="J20" s="28" t="inlineStr">
         <is>
-          <t>K&amp;H Thermo-Pond 3.0 Floating De-Icer, 100W</t>
+          <t>K&amp;H Thermo-Pond 3.0 Floating Pond De-Icer, 100W</t>
         </is>
       </c>
       <c r="K20" s="29" t="inlineStr">
@@ -1632,11 +1672,19 @@
         </is>
       </c>
       <c r="P20" s="31" t="n"/>
-      <c r="Q20" s="29" t="n"/>
-      <c r="R20" s="32" t="n"/>
+      <c r="Q20" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R20" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="S20" s="28" t="inlineStr">
         <is>
-          <t>Sourced 2026-09-28 from Amazon search results; price not visible from here. Rated for ponds up to 1,000 gal per listing snippet. Alt: TURBRO PD400A 400W (B0CHF46RK7), more power than needed.</t>
+          <t>Catalog slug: pond-deicer-kh-thermo-pond-100w. Sourced 2026-09-28 from Amazon search results; price not visible from here. Rated for ponds up to 1,000 gal per listing snippet. Alt: TURBRO PD400A 400W (B0CHF46RK7), more power than needed.</t>
         </is>
       </c>
     </row>
@@ -1677,12 +1725,12 @@
       <c r="H21" s="28" t="inlineStr"/>
       <c r="I21" s="29" t="inlineStr">
         <is>
-          <t>Link found</t>
+          <t>Added to catalog</t>
         </is>
       </c>
       <c r="J21" s="28" t="inlineStr">
         <is>
-          <t>Flexwatt Reptile Heat Tape, 6 in, 10 ft roll</t>
+          <t>Flexwatt Reptile Heat Tape, 6 in, 10 ft Roll</t>
         </is>
       </c>
       <c r="K21" s="29" t="inlineStr">
@@ -1710,11 +1758,19 @@
         </is>
       </c>
       <c r="P21" s="31" t="n"/>
-      <c r="Q21" s="29" t="n"/>
-      <c r="R21" s="32" t="n"/>
+      <c r="Q21" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R21" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="S21" s="28" t="inlineStr">
         <is>
-          <t>Sourced 2026-09-28 from Amazon search results; price not visible from here. Needs a thermostat (catalog already has several). Several Flexwatt listings are sold by the foot. Alt: 11 in x 3 ft Flexwatt (B00BO0MKNA).</t>
+          <t>Catalog slug: heat-tape-flexwatt-6in-10ft. Sourced 2026-09-28 from Amazon search results; price not visible from here. Needs a thermostat (catalog already has several). Several Flexwatt listings are sold by the foot. Alt: 11 in x 3 ft Flexwatt (B00BO0MKNA).</t>
         </is>
       </c>
     </row>
@@ -1755,12 +1811,12 @@
       <c r="H22" s="28" t="inlineStr"/>
       <c r="I22" s="29" t="inlineStr">
         <is>
-          <t>Link found</t>
+          <t>Added to catalog</t>
         </is>
       </c>
       <c r="J22" s="28" t="inlineStr">
         <is>
-          <t>BN-LINK 24-Hour Mechanical Outlet Timer, 1-Pack</t>
+          <t>BN-LINK 24-Hour Mechanical Outlet Timer</t>
         </is>
       </c>
       <c r="K22" s="29" t="inlineStr">
@@ -1788,11 +1844,19 @@
         </is>
       </c>
       <c r="P22" s="31" t="n"/>
-      <c r="Q22" s="29" t="n"/>
-      <c r="R22" s="32" t="n"/>
+      <c r="Q22" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R22" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="S22" s="28" t="inlineStr">
         <is>
-          <t>Sourced 2026-09-28 from Amazon search results; price not visible from here. Alt: BN-LINK dual outlet mechanical timer (B00MVEMD76); 2-pack B074927BKZ.</t>
+          <t>Catalog slug: outlet-timer-bn-link-mechanical. Sourced 2026-09-28 from Amazon search results; price not visible from here. Alt: BN-LINK dual outlet mechanical timer (B00MVEMD76); 2-pack B074927BKZ.</t>
         </is>
       </c>
     </row>
@@ -1837,7 +1901,7 @@
       </c>
       <c r="I23" s="29" t="inlineStr">
         <is>
-          <t>Link found</t>
+          <t>Added to catalog</t>
         </is>
       </c>
       <c r="J23" s="28" t="inlineStr">
@@ -1870,11 +1934,19 @@
         </is>
       </c>
       <c r="P23" s="31" t="n"/>
-      <c r="Q23" s="29" t="n"/>
-      <c r="R23" s="32" t="n"/>
+      <c r="Q23" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R23" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="S23" s="28" t="inlineStr">
         <is>
-          <t>Sourced 2026-09-28 from Amazon search results; price not visible from here. Second pick: Hikari Bio-Pure Freeze Dried Brine Shrimp 0.42 oz (B00025K1HK). Daphnia: Hikari Bio-Pure FD Daphnia (B003WRG54I). Freeze-dried chosen because frozen does not ship well.</t>
+          <t>Catalog slug: freeze-dried-bloodworms-omega-one, freeze-dried-brine-shrimp-hikari. Also added: Hikari Bio-Pure Freeze Dried Brine Shrimp, 0.42 oz (https://www.amazon.com/dp/B00025K1HK). Sourced 2026-09-28 from Amazon search results; price not visible from here. Second pick: Hikari Bio-Pure Freeze Dried Brine Shrimp 0.42 oz (B00025K1HK). Daphnia: Hikari Bio-Pure FD Daphnia (B003WRG54I). Freeze-dried chosen because frozen does not ship well.</t>
         </is>
       </c>
     </row>
@@ -1915,12 +1987,12 @@
       <c r="H24" s="28" t="inlineStr"/>
       <c r="I24" s="29" t="inlineStr">
         <is>
-          <t>Link found</t>
+          <t>Added to catalog</t>
         </is>
       </c>
       <c r="J24" s="28" t="inlineStr">
         <is>
-          <t>Josh's Frogs Organic Magnolia Leaf Litter, 1 gal</t>
+          <t>Josh's Frogs Organic Magnolia Leaf Litter, 1 Gallon</t>
         </is>
       </c>
       <c r="K24" s="29" t="inlineStr">
@@ -1948,11 +2020,19 @@
         </is>
       </c>
       <c r="P24" s="31" t="n"/>
-      <c r="Q24" s="29" t="n"/>
-      <c r="R24" s="32" t="n"/>
+      <c r="Q24" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R24" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="S24" s="28" t="inlineStr">
         <is>
-          <t>Sourced 2026-09-28 from Amazon search results; price not visible from here. Alt: Galapagos Magnolia Leaf Litter 4 qt (B087WJF92B). No oak listing found.</t>
+          <t>Catalog slug: leaf-litter-joshs-frogs-magnolia. Sourced 2026-09-28 from Amazon search results; price not visible from here. Alt: Galapagos Magnolia Leaf Litter 4 qt (B087WJF92B). No oak listing found.</t>
         </is>
       </c>
     </row>
@@ -1997,12 +2077,12 @@
       </c>
       <c r="I25" s="29" t="inlineStr">
         <is>
-          <t>Link found</t>
+          <t>Added to catalog</t>
         </is>
       </c>
       <c r="J25" s="28" t="inlineStr">
         <is>
-          <t>NICREW ClassicLED, 36 to 48 in, 25W</t>
+          <t>NICREW ClassicLED Aquarium Light, 36 to 48 in</t>
         </is>
       </c>
       <c r="K25" s="29" t="inlineStr">
@@ -2030,11 +2110,19 @@
         </is>
       </c>
       <c r="P25" s="31" t="n"/>
-      <c r="Q25" s="29" t="n"/>
-      <c r="R25" s="32" t="n"/>
+      <c r="Q25" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R25" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="S25" s="28" t="inlineStr">
         <is>
-          <t>Sourced 2026-09-28 from Amazon search results; price not visible from here. Size must match the tank. Same line: 28 to 36 in (B01C84SLRO). ClassicLED Plus: 18-24 in (B07F7391M2), 30-36 in (B07F6XD2FH), 48-54 in (B07KK6G8ZL).</t>
+          <t>Catalog slug: aquarium-led-nicrew-classicled-36-48. Sourced 2026-09-28 from Amazon search results; price not visible from here. Size must match the tank. Same line: 28 to 36 in (B01C84SLRO). ClassicLED Plus: 18-24 in (B07F7391M2), 30-36 in (B07F6XD2FH), 48-54 in (B07KK6G8ZL).</t>
         </is>
       </c>
     </row>
@@ -2079,12 +2167,12 @@
       </c>
       <c r="I26" s="29" t="inlineStr">
         <is>
-          <t>Link found</t>
+          <t>Added to catalog</t>
         </is>
       </c>
       <c r="J26" s="28" t="inlineStr">
         <is>
-          <t>Sterilite 32 Qt Latching Storage Box, clear</t>
+          <t>Sterilite 32 Qt Latching Storage Box</t>
         </is>
       </c>
       <c r="K26" s="29" t="inlineStr">
@@ -2112,11 +2200,19 @@
         </is>
       </c>
       <c r="P26" s="31" t="n"/>
-      <c r="Q26" s="29" t="n"/>
-      <c r="R26" s="32" t="n"/>
+      <c r="Q26" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R26" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="S26" s="28" t="inlineStr">
         <is>
-          <t>Sourced 2026-09-28 from Amazon search results; price not visible from here. Larger: Sterilite 16598008 56 Qt Storage Box (B00C9MR9YM). Latching 56 qt only found as an 8-pack (B084Z789LQ).</t>
+          <t>Catalog slug: storage-tub-sterilite-32qt-latching, storage-tub-sterilite-56qt. Also added: Sterilite 56 Qt Storage Box (https://www.amazon.com/dp/B00C9MR9YM). Sourced 2026-09-28 from Amazon search results; price not visible from here. Larger: Sterilite 16598008 56 Qt Storage Box (B00C9MR9YM). Latching 56 qt only found as an 8-pack (B084Z789LQ).</t>
         </is>
       </c>
     </row>
@@ -2161,12 +2257,12 @@
       </c>
       <c r="I27" s="29" t="inlineStr">
         <is>
-          <t>Link found</t>
+          <t>Added to catalog</t>
         </is>
       </c>
       <c r="J27" s="28" t="inlineStr">
         <is>
-          <t>BirdCageLiners 100 Pre-Cut Sheets, 40 lb kraft (medium cages)</t>
+          <t>BirdCageLiners Pre-Cut Kraft Paper Sheets, 100 Pack</t>
         </is>
       </c>
       <c r="K27" s="29" t="inlineStr">
@@ -2194,11 +2290,19 @@
         </is>
       </c>
       <c r="P27" s="31" t="n"/>
-      <c r="Q27" s="29" t="n"/>
-      <c r="R27" s="32" t="n"/>
+      <c r="Q27" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R27" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="S27" s="28" t="inlineStr">
         <is>
-          <t>Sourced 2026-09-28 from Amazon search results; price not visible from here. Snippet says no ink, dyes or wax. Roll alt: The Paper Factory brown butcher paper 17.75 in x 100 ft (B08D6W7DS3). Unprinted newsprint alt: VIOLETTO 120 sheets (B0GVJCGYNX).</t>
+          <t>Catalog slug: cage-liner-birdcageliners-precut-kraft. Sourced 2026-09-28 from Amazon search results; price not visible from here. Snippet says no ink, dyes or wax. Roll alt: The Paper Factory brown butcher paper 17.75 in x 100 ft (B08D6W7DS3). Unprinted newsprint alt: VIOLETTO 120 sheets (B0GVJCGYNX).</t>
         </is>
       </c>
     </row>
@@ -2239,12 +2343,12 @@
       <c r="H28" s="28" t="inlineStr"/>
       <c r="I28" s="29" t="inlineStr">
         <is>
-          <t>Link found</t>
+          <t>Added to catalog</t>
         </is>
       </c>
       <c r="J28" s="28" t="inlineStr">
         <is>
-          <t>LIXIT Chew Proof Glass Water Bottle 16 oz</t>
+          <t>LIXIT Chew Proof Glass Water Bottle, 16 oz</t>
         </is>
       </c>
       <c r="K28" s="29" t="inlineStr">
@@ -2272,11 +2376,19 @@
         </is>
       </c>
       <c r="P28" s="31" t="n"/>
-      <c r="Q28" s="29" t="n"/>
-      <c r="R28" s="32" t="n"/>
+      <c r="Q28" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R28" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="S28" s="28" t="inlineStr">
         <is>
-          <t>Sourced 2026-09-28 from Amazon search results; price not visible from here. Alt: Exotic Nutrition hanging glass bottle 12 oz (B0763P4H2L), good for smaller rodents.</t>
+          <t>Catalog slug: water-bottle-lixit-glass-16oz. Sourced 2026-09-28 from Amazon search results; price not visible from here. Alt: Exotic Nutrition hanging glass bottle 12 oz (B0763P4H2L), good for smaller rodents.</t>
         </is>
       </c>
     </row>
@@ -2317,12 +2429,12 @@
       <c r="H29" s="28" t="inlineStr"/>
       <c r="I29" s="29" t="inlineStr">
         <is>
-          <t>Link found</t>
+          <t>Added to catalog</t>
         </is>
       </c>
       <c r="J29" s="28" t="inlineStr">
         <is>
-          <t>Zoo Med ReptiSoil 10 qt</t>
+          <t>Michigan Peat Garden Magic Top Soil Blend, 40 lb</t>
         </is>
       </c>
       <c r="K29" s="29" t="inlineStr">
@@ -2332,7 +2444,7 @@
       </c>
       <c r="L29" s="28" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/dp/B01MFA1RM7</t>
+          <t>https://www.amazon.com/dp/B000GQ4KX6</t>
         </is>
       </c>
       <c r="M29" s="30">
@@ -2341,20 +2453,28 @@
       </c>
       <c r="N29" s="28" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/dp/B01MFA1RM7?tag=beastlyfacts-20</t>
+          <t>https://www.amazon.com/dp/B000GQ4KX6?tag=beastlyfacts-20</t>
         </is>
       </c>
       <c r="O29" s="29" t="inlineStr">
         <is>
-          <t>check</t>
+          <t>$28.99 (seen 09-28)</t>
         </is>
       </c>
       <c r="P29" s="31" t="n"/>
-      <c r="Q29" s="29" t="n"/>
-      <c r="R29" s="32" t="n"/>
+      <c r="Q29" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R29" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="S29" s="28" t="inlineStr">
         <is>
-          <t>Sourced 2026-09-28 from Amazon search results; price not visible from here. Reptile soil blend (peat, soil, sand, carbon), not plain topsoil. No plain organic topsoil listing found. Alt: Josh's Frogs BioBedding Tropical 4 qt (B086R65X96). Confirm no added fertilizer on the page.</t>
+          <t>Catalog slug: topsoil-michigan-peat-garden-magic-40lb. Owner pick, replaces the earlier ReptiSoil suggestion.</t>
         </is>
       </c>
     </row>
@@ -2395,7 +2515,7 @@
       <c r="H30" s="28" t="inlineStr"/>
       <c r="I30" s="29" t="inlineStr">
         <is>
-          <t>Link found</t>
+          <t>Added to catalog</t>
         </is>
       </c>
       <c r="J30" s="28" t="inlineStr">
@@ -2428,11 +2548,19 @@
         </is>
       </c>
       <c r="P30" s="31" t="n"/>
-      <c r="Q30" s="29" t="n"/>
-      <c r="R30" s="32" t="n"/>
+      <c r="Q30" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R30" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="S30" s="28" t="inlineStr">
         <is>
-          <t>Sourced 2026-09-28 from Amazon search results; price not visible from here. Title confirmed on the product page. Alt: Rep-Cal Phosphorus-Free Calcium without D3, 4.1 oz (B00BS96GLE).</t>
+          <t>Catalog slug: calcium-zoo-med-without-d3. Sourced 2026-09-28 from Amazon search results; price not visible from here. Title confirmed on the product page. Alt: Rep-Cal Phosphorus-Free Calcium without D3, 4.1 oz (B00BS96GLE).</t>
         </is>
       </c>
     </row>
@@ -2477,12 +2605,12 @@
       </c>
       <c r="I31" s="29" t="inlineStr">
         <is>
-          <t>Link found</t>
+          <t>Added to catalog</t>
         </is>
       </c>
       <c r="J31" s="28" t="inlineStr">
         <is>
-          <t>Aqueon 40 Gallon Breeder Tank, 36x18x16</t>
+          <t>Aqueon 40 Gallon Breeder Tank, 36x18x16 in</t>
         </is>
       </c>
       <c r="K31" s="29" t="inlineStr">
@@ -2510,11 +2638,19 @@
         </is>
       </c>
       <c r="P31" s="31" t="n"/>
-      <c r="Q31" s="29" t="n"/>
-      <c r="R31" s="32" t="n"/>
+      <c r="Q31" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R31" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="S31" s="28" t="inlineStr">
         <is>
-          <t>Sourced 2026-09-28 from Amazon search results; price not visible from here. Alt: Perfecto 40 gal breeder 36x18x16 (B004HSULOG). Big tanks sometimes ship poorly; check availability.</t>
+          <t>Catalog slug: tank-aqueon-40-breeder. Sourced 2026-09-28 from Amazon search results; price not visible from here. Alt: Perfecto 40 gal breeder 36x18x16 (B004HSULOG). Big tanks sometimes ship poorly; check availability.</t>
         </is>
       </c>
     </row>
@@ -2555,12 +2691,12 @@
       <c r="H32" s="28" t="inlineStr"/>
       <c r="I32" s="29" t="inlineStr">
         <is>
-          <t>Link found</t>
+          <t>Added to catalog</t>
         </is>
       </c>
       <c r="J32" s="28" t="inlineStr">
         <is>
-          <t>Prevue Universal Bird Cage Cover, Medium (12502)</t>
+          <t>Prevue Universal Bird Cage Cover, Medium</t>
         </is>
       </c>
       <c r="K32" s="29" t="inlineStr">
@@ -2588,11 +2724,19 @@
         </is>
       </c>
       <c r="P32" s="31" t="n"/>
-      <c r="Q32" s="29" t="n"/>
-      <c r="R32" s="32" t="n"/>
+      <c r="Q32" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R32" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="S32" s="28" t="inlineStr">
         <is>
-          <t>Sourced 2026-09-28 from Amazon search results; price not visible from here. Medium fits cages up to 20x20x29 in. Larger: Prevue Good Night cover (B0002AQ5ZC), title says both Extra Large and Large, check the size.</t>
+          <t>Catalog slug: cage-cover-prevue-universal-medium. Sourced 2026-09-28 from Amazon search results; price not visible from here. Medium fits cages up to 20x20x29 in. Larger: Prevue Good Night cover (B0002AQ5ZC), title says both Extra Large and Large, check the size.</t>
         </is>
       </c>
     </row>
@@ -2633,7 +2777,7 @@
       <c r="H33" s="28" t="inlineStr"/>
       <c r="I33" s="29" t="inlineStr">
         <is>
-          <t>Link found</t>
+          <t>Added to catalog</t>
         </is>
       </c>
       <c r="J33" s="28" t="inlineStr">
@@ -2666,11 +2810,19 @@
         </is>
       </c>
       <c r="P33" s="31" t="n"/>
-      <c r="Q33" s="29" t="n"/>
-      <c r="R33" s="32" t="n"/>
+      <c r="Q33" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R33" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="S33" s="28" t="inlineStr">
         <is>
-          <t>Sourced 2026-09-28 from Amazon search results; price not visible from here. Title confirmed on the product page. Smaller: 200 ml (B00ECJ5NIY). Do not use F10SCXD listings (with detergent).</t>
+          <t>Catalog slug: disinfectant-f10sc-concentrate-1l. Sourced 2026-09-28 from Amazon search results; price not visible from here. Title confirmed on the product page. Smaller: 200 ml (B00ECJ5NIY). Do not use F10SCXD listings (with detergent).</t>
         </is>
       </c>
     </row>
@@ -2711,22 +2863,54 @@
       <c r="H34" s="28" t="inlineStr"/>
       <c r="I34" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J34" s="28" t="n"/>
-      <c r="K34" s="29" t="n"/>
-      <c r="L34" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J34" s="28" t="inlineStr">
+        <is>
+          <t>Espoma Organic Sphagnum Peat Moss</t>
+        </is>
+      </c>
+      <c r="K34" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L34" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0037AP20I</t>
+        </is>
+      </c>
       <c r="M34" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L34)),MID(L34,SEARCH("/dp/",L34)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N34" s="28" t="n"/>
-      <c r="O34" s="29" t="n"/>
+      <c r="N34" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0037AP20I?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O34" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P34" s="31" t="n"/>
-      <c r="Q34" s="29" t="n"/>
-      <c r="R34" s="32" t="n"/>
-      <c r="S34" s="28" t="n"/>
+      <c r="Q34" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R34" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S34" s="28" t="inlineStr">
+        <is>
+          <t>Catalog slug: peat-moss-espoma-organic.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="41" t="inlineStr">
@@ -2769,22 +2953,54 @@
       </c>
       <c r="I35" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J35" s="28" t="n"/>
-      <c r="K35" s="29" t="n"/>
-      <c r="L35" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J35" s="28" t="inlineStr">
+        <is>
+          <t>Oxbow Orchard Grass Hay, 40 oz</t>
+        </is>
+      </c>
+      <c r="K35" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L35" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B000WFKP80</t>
+        </is>
+      </c>
       <c r="M35" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L35)),MID(L35,SEARCH("/dp/",L35)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N35" s="28" t="n"/>
-      <c r="O35" s="29" t="n"/>
+      <c r="N35" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B000WFKP80?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O35" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P35" s="31" t="n"/>
-      <c r="Q35" s="29" t="n"/>
-      <c r="R35" s="32" t="n"/>
-      <c r="S35" s="28" t="n"/>
+      <c r="Q35" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R35" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S35" s="28" t="inlineStr">
+        <is>
+          <t>Catalog slug: hay-oxbow-orchard-40oz.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="41" t="inlineStr">
@@ -2823,22 +3039,54 @@
       <c r="H36" s="28" t="inlineStr"/>
       <c r="I36" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J36" s="28" t="n"/>
-      <c r="K36" s="29" t="n"/>
-      <c r="L36" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J36" s="28" t="inlineStr">
+        <is>
+          <t>Kaytee Clean &amp; Cozy Paper Bedding, White, 49.2 L</t>
+        </is>
+      </c>
+      <c r="K36" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L36" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B007R6G8JW</t>
+        </is>
+      </c>
       <c r="M36" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L36)),MID(L36,SEARCH("/dp/",L36)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N36" s="28" t="n"/>
-      <c r="O36" s="29" t="n"/>
+      <c r="N36" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B007R6G8JW?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O36" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P36" s="31" t="n"/>
-      <c r="Q36" s="29" t="n"/>
-      <c r="R36" s="32" t="n"/>
-      <c r="S36" s="28" t="n"/>
+      <c r="Q36" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R36" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S36" s="28" t="inlineStr">
+        <is>
+          <t>Catalog slug: bedding-kaytee-clean-cozy-white.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="41" t="inlineStr">
@@ -2877,22 +3125,54 @@
       <c r="H37" s="28" t="inlineStr"/>
       <c r="I37" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J37" s="28" t="n"/>
-      <c r="K37" s="29" t="n"/>
-      <c r="L37" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J37" s="28" t="inlineStr">
+        <is>
+          <t>Omega One Veggie Kelp Flakes, 2.2 oz</t>
+        </is>
+      </c>
+      <c r="K37" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L37" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0046HIG7W</t>
+        </is>
+      </c>
       <c r="M37" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L37)),MID(L37,SEARCH("/dp/",L37)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N37" s="28" t="n"/>
-      <c r="O37" s="29" t="n"/>
+      <c r="N37" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0046HIG7W?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O37" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P37" s="31" t="n"/>
-      <c r="Q37" s="29" t="n"/>
-      <c r="R37" s="32" t="n"/>
-      <c r="S37" s="28" t="n"/>
+      <c r="Q37" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R37" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S37" s="28" t="inlineStr">
+        <is>
+          <t>Catalog slug: fish-food-omega-one-veggie-kelp-flakes.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="41" t="inlineStr">
@@ -2931,22 +3211,54 @@
       <c r="H38" s="28" t="inlineStr"/>
       <c r="I38" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J38" s="28" t="n"/>
-      <c r="K38" s="29" t="n"/>
-      <c r="L38" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J38" s="28" t="inlineStr">
+        <is>
+          <t>CaribSea Crushed Coral, 10 lb</t>
+        </is>
+      </c>
+      <c r="K38" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L38" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B000ELY1YQ</t>
+        </is>
+      </c>
       <c r="M38" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L38)),MID(L38,SEARCH("/dp/",L38)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N38" s="28" t="n"/>
-      <c r="O38" s="29" t="n"/>
+      <c r="N38" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B000ELY1YQ?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O38" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P38" s="31" t="n"/>
-      <c r="Q38" s="29" t="n"/>
-      <c r="R38" s="32" t="n"/>
-      <c r="S38" s="28" t="n"/>
+      <c r="Q38" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R38" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S38" s="28" t="inlineStr">
+        <is>
+          <t>Catalog slug: crushed-coral-caribsea-10lb.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="41" t="inlineStr">
@@ -2985,22 +3297,54 @@
       <c r="H39" s="28" t="inlineStr"/>
       <c r="I39" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J39" s="28" t="n"/>
-      <c r="K39" s="29" t="n"/>
-      <c r="L39" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J39" s="28" t="inlineStr">
+        <is>
+          <t>SunGrow Indian Almond Leaves (Catappa), 50 Pack</t>
+        </is>
+      </c>
+      <c r="K39" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L39" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B01G78H5XS</t>
+        </is>
+      </c>
       <c r="M39" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L39)),MID(L39,SEARCH("/dp/",L39)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N39" s="28" t="n"/>
-      <c r="O39" s="29" t="n"/>
+      <c r="N39" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B01G78H5XS?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O39" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P39" s="31" t="n"/>
-      <c r="Q39" s="29" t="n"/>
-      <c r="R39" s="32" t="n"/>
-      <c r="S39" s="28" t="n"/>
+      <c r="Q39" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R39" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S39" s="28" t="inlineStr">
+        <is>
+          <t>Catalog slug: catappa-leaves-sungrow-50.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="41" t="inlineStr">
@@ -3039,22 +3383,54 @@
       <c r="H40" s="28" t="inlineStr"/>
       <c r="I40" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J40" s="28" t="n"/>
-      <c r="K40" s="29" t="n"/>
-      <c r="L40" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J40" s="28" t="inlineStr">
+        <is>
+          <t>Salty Shrimp Mineral GH/KH+, 200 g</t>
+        </is>
+      </c>
+      <c r="K40" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L40" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B00HZLUGSI</t>
+        </is>
+      </c>
       <c r="M40" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L40)),MID(L40,SEARCH("/dp/",L40)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N40" s="28" t="n"/>
-      <c r="O40" s="29" t="n"/>
+      <c r="N40" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B00HZLUGSI?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O40" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P40" s="31" t="n"/>
-      <c r="Q40" s="29" t="n"/>
-      <c r="R40" s="32" t="n"/>
-      <c r="S40" s="28" t="n"/>
+      <c r="Q40" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R40" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S40" s="28" t="inlineStr">
+        <is>
+          <t>Catalog slug: shrimp-mineral-salty-shrimp-gh-kh, shrimp-mineral-salty-shrimp-gh. Also added: Salty Shrimp Bee Shrimp Mineral GH+, 110 g (https://www.amazon.com/dp/B06Y5M7CGB).</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="41" t="inlineStr">
@@ -3093,22 +3469,54 @@
       <c r="H41" s="28" t="inlineStr"/>
       <c r="I41" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J41" s="28" t="n"/>
-      <c r="K41" s="29" t="n"/>
-      <c r="L41" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J41" s="28" t="inlineStr">
+        <is>
+          <t>Mazuri Rat &amp; Mouse Diet Lab Blocks, 2 lb</t>
+        </is>
+      </c>
+      <c r="K41" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L41" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B00JR8K8DA</t>
+        </is>
+      </c>
       <c r="M41" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L41)),MID(L41,SEARCH("/dp/",L41)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N41" s="28" t="n"/>
-      <c r="O41" s="29" t="n"/>
+      <c r="N41" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B00JR8K8DA?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O41" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P41" s="31" t="n"/>
-      <c r="Q41" s="29" t="n"/>
-      <c r="R41" s="32" t="n"/>
-      <c r="S41" s="28" t="n"/>
+      <c r="Q41" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R41" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S41" s="28" t="inlineStr">
+        <is>
+          <t>Catalog slug: rat-block-mazuri-2lb.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="41" t="inlineStr">
@@ -3147,22 +3555,54 @@
       <c r="H42" s="28" t="inlineStr"/>
       <c r="I42" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J42" s="28" t="n"/>
-      <c r="K42" s="29" t="n"/>
-      <c r="L42" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J42" s="28" t="inlineStr">
+        <is>
+          <t>Manna Pro Crushed Oyster Shell, 5 lb</t>
+        </is>
+      </c>
+      <c r="K42" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L42" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B000MD59TC</t>
+        </is>
+      </c>
       <c r="M42" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L42)),MID(L42,SEARCH("/dp/",L42)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N42" s="28" t="n"/>
-      <c r="O42" s="29" t="n"/>
+      <c r="N42" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B000MD59TC?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O42" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P42" s="31" t="n"/>
-      <c r="Q42" s="29" t="n"/>
-      <c r="R42" s="32" t="n"/>
-      <c r="S42" s="28" t="n"/>
+      <c r="Q42" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R42" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S42" s="28" t="inlineStr">
+        <is>
+          <t>Catalog slug: oyster-shell-manna-pro-5lb.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="41" t="inlineStr">
@@ -3201,22 +3641,54 @@
       <c r="H43" s="28" t="inlineStr"/>
       <c r="I43" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J43" s="28" t="n"/>
-      <c r="K43" s="29" t="n"/>
-      <c r="L43" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J43" s="28" t="inlineStr">
+        <is>
+          <t>Higgins Protein Egg Food, 5 oz (3 Pack)</t>
+        </is>
+      </c>
+      <c r="K43" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L43" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B07P9VFYVW</t>
+        </is>
+      </c>
       <c r="M43" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L43)),MID(L43,SEARCH("/dp/",L43)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N43" s="28" t="n"/>
-      <c r="O43" s="29" t="n"/>
+      <c r="N43" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B07P9VFYVW?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O43" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P43" s="31" t="n"/>
-      <c r="Q43" s="29" t="n"/>
-      <c r="R43" s="32" t="n"/>
-      <c r="S43" s="28" t="n"/>
+      <c r="Q43" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R43" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S43" s="28" t="inlineStr">
+        <is>
+          <t>Catalog slug: egg-food-higgins-3pack.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="41" t="inlineStr">
@@ -3255,22 +3727,54 @@
       <c r="H44" s="28" t="inlineStr"/>
       <c r="I44" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J44" s="28" t="n"/>
-      <c r="K44" s="29" t="n"/>
-      <c r="L44" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J44" s="28" t="inlineStr">
+        <is>
+          <t>Repashy SuperFoods Vitamin A Plus, 3 oz</t>
+        </is>
+      </c>
+      <c r="K44" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L44" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0D6D8XYLV</t>
+        </is>
+      </c>
       <c r="M44" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L44)),MID(L44,SEARCH("/dp/",L44)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N44" s="28" t="n"/>
-      <c r="O44" s="29" t="n"/>
+      <c r="N44" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0D6D8XYLV?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O44" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P44" s="31" t="n"/>
-      <c r="Q44" s="29" t="n"/>
-      <c r="R44" s="32" t="n"/>
-      <c r="S44" s="28" t="n"/>
+      <c r="Q44" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R44" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S44" s="28" t="inlineStr">
+        <is>
+          <t>Catalog slug: vitamin-repashy-vitamin-a-plus.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="41" t="inlineStr">
@@ -3309,22 +3813,54 @@
       <c r="H45" s="28" t="inlineStr"/>
       <c r="I45" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J45" s="28" t="n"/>
-      <c r="K45" s="29" t="n"/>
-      <c r="L45" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J45" s="28" t="inlineStr">
+        <is>
+          <t>Oxbow Eco Straw Pelleted Litter, 20 lb</t>
+        </is>
+      </c>
+      <c r="K45" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L45" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0017JGBAQ</t>
+        </is>
+      </c>
       <c r="M45" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L45)),MID(L45,SEARCH("/dp/",L45)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N45" s="28" t="n"/>
-      <c r="O45" s="29" t="n"/>
+      <c r="N45" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0017JGBAQ?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O45" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P45" s="31" t="n"/>
-      <c r="Q45" s="29" t="n"/>
-      <c r="R45" s="32" t="n"/>
-      <c r="S45" s="28" t="n"/>
+      <c r="Q45" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R45" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S45" s="28" t="inlineStr">
+        <is>
+          <t>Catalog slug: litter-oxbow-eco-straw-20lb.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="41" t="inlineStr">
@@ -3363,22 +3899,54 @@
       <c r="H46" s="28" t="inlineStr"/>
       <c r="I46" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J46" s="28" t="n"/>
-      <c r="K46" s="29" t="n"/>
-      <c r="L46" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J46" s="28" t="inlineStr">
+        <is>
+          <t>Hikari Betta Bio-Gold, 0.70 oz</t>
+        </is>
+      </c>
+      <c r="K46" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L46" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B00025Z74C</t>
+        </is>
+      </c>
       <c r="M46" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L46)),MID(L46,SEARCH("/dp/",L46)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N46" s="28" t="n"/>
-      <c r="O46" s="29" t="n"/>
+      <c r="N46" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B00025Z74C?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O46" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P46" s="31" t="n"/>
-      <c r="Q46" s="29" t="n"/>
-      <c r="R46" s="32" t="n"/>
-      <c r="S46" s="28" t="n"/>
+      <c r="Q46" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R46" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S46" s="28" t="inlineStr">
+        <is>
+          <t>Catalog slug: betta-food-hikari-bio-gold.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="41" t="inlineStr">
@@ -3417,22 +3985,54 @@
       <c r="H47" s="28" t="inlineStr"/>
       <c r="I47" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J47" s="28" t="n"/>
-      <c r="K47" s="29" t="n"/>
-      <c r="L47" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J47" s="28" t="inlineStr">
+        <is>
+          <t>Zoo Med Hermit Crab Food</t>
+        </is>
+      </c>
+      <c r="K47" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L47" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B00027ZVDM</t>
+        </is>
+      </c>
       <c r="M47" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L47)),MID(L47,SEARCH("/dp/",L47)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N47" s="28" t="n"/>
-      <c r="O47" s="29" t="n"/>
+      <c r="N47" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B00027ZVDM?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O47" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P47" s="31" t="n"/>
-      <c r="Q47" s="29" t="n"/>
-      <c r="R47" s="32" t="n"/>
-      <c r="S47" s="28" t="n"/>
+      <c r="Q47" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R47" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S47" s="28" t="inlineStr">
+        <is>
+          <t>Catalog slug: hermit-crab-food-zoo-med.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="41" t="inlineStr">
@@ -3471,22 +4071,54 @@
       <c r="H48" s="28" t="inlineStr"/>
       <c r="I48" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J48" s="28" t="n"/>
-      <c r="K48" s="29" t="n"/>
-      <c r="L48" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J48" s="28" t="inlineStr">
+        <is>
+          <t>Josh's Frogs Roach Rations, 1 Gallon</t>
+        </is>
+      </c>
+      <c r="K48" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L48" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B01MZH5FFU</t>
+        </is>
+      </c>
       <c r="M48" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L48)),MID(L48,SEARCH("/dp/",L48)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N48" s="28" t="n"/>
-      <c r="O48" s="29" t="n"/>
+      <c r="N48" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B01MZH5FFU?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O48" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P48" s="31" t="n"/>
-      <c r="Q48" s="29" t="n"/>
-      <c r="R48" s="32" t="n"/>
-      <c r="S48" s="28" t="n"/>
+      <c r="Q48" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R48" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S48" s="28" t="inlineStr">
+        <is>
+          <t>Catalog slug: roach-food-joshs-frogs-roach-rations.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="41" t="inlineStr">
@@ -3525,22 +4157,54 @@
       <c r="H49" s="28" t="inlineStr"/>
       <c r="I49" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J49" s="28" t="n"/>
-      <c r="K49" s="29" t="n"/>
-      <c r="L49" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J49" s="28" t="inlineStr">
+        <is>
+          <t>Hikari Discus Bio-Gold, 2.82 oz</t>
+        </is>
+      </c>
+      <c r="K49" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L49" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B00025JZBS</t>
+        </is>
+      </c>
       <c r="M49" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L49)),MID(L49,SEARCH("/dp/",L49)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N49" s="28" t="n"/>
-      <c r="O49" s="29" t="n"/>
+      <c r="N49" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B00025JZBS?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O49" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P49" s="31" t="n"/>
-      <c r="Q49" s="29" t="n"/>
-      <c r="R49" s="32" t="n"/>
-      <c r="S49" s="28" t="n"/>
+      <c r="Q49" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R49" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S49" s="28" t="inlineStr">
+        <is>
+          <t>Catalog slug: discus-food-hikari-bio-gold.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="41" t="inlineStr">
@@ -3579,22 +4243,54 @@
       <c r="H50" s="28" t="inlineStr"/>
       <c r="I50" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J50" s="28" t="n"/>
-      <c r="K50" s="29" t="n"/>
-      <c r="L50" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J50" s="28" t="inlineStr">
+        <is>
+          <t>Higgins Vita Seed Finch Food, 25 lb</t>
+        </is>
+      </c>
+      <c r="K50" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L50" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B00E1JOYEY</t>
+        </is>
+      </c>
       <c r="M50" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L50)),MID(L50,SEARCH("/dp/",L50)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N50" s="28" t="n"/>
-      <c r="O50" s="29" t="n"/>
+      <c r="N50" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B00E1JOYEY?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O50" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P50" s="31" t="n"/>
-      <c r="Q50" s="29" t="n"/>
-      <c r="R50" s="32" t="n"/>
-      <c r="S50" s="28" t="n"/>
+      <c r="Q50" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R50" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S50" s="28" t="inlineStr">
+        <is>
+          <t>Catalog slug: finch-seed-higgins-vita-25lb.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="41" t="inlineStr">
@@ -3633,22 +4329,54 @@
       <c r="H51" s="28" t="inlineStr"/>
       <c r="I51" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J51" s="28" t="n"/>
-      <c r="K51" s="29" t="n"/>
-      <c r="L51" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J51" s="28" t="inlineStr">
+        <is>
+          <t>Oxbow Essentials Adult Guinea Pig Food, 10 lb</t>
+        </is>
+      </c>
+      <c r="K51" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L51" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0017JFIDC</t>
+        </is>
+      </c>
       <c r="M51" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L51)),MID(L51,SEARCH("/dp/",L51)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N51" s="28" t="n"/>
-      <c r="O51" s="29" t="n"/>
+      <c r="N51" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0017JFIDC?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O51" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P51" s="31" t="n"/>
-      <c r="Q51" s="29" t="n"/>
-      <c r="R51" s="32" t="n"/>
-      <c r="S51" s="28" t="n"/>
+      <c r="Q51" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R51" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S51" s="28" t="inlineStr">
+        <is>
+          <t>Catalog slug: guinea-pig-food-oxbow-essentials-adult.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="41" t="inlineStr">
@@ -3687,22 +4415,54 @@
       <c r="H52" s="28" t="inlineStr"/>
       <c r="I52" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J52" s="28" t="n"/>
-      <c r="K52" s="29" t="n"/>
-      <c r="L52" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J52" s="28" t="inlineStr">
+        <is>
+          <t>Exotic Nutrition Hedgehog Complete, 2 lb</t>
+        </is>
+      </c>
+      <c r="K52" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L52" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B01HOYD69Q</t>
+        </is>
+      </c>
       <c r="M52" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L52)),MID(L52,SEARCH("/dp/",L52)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N52" s="28" t="n"/>
-      <c r="O52" s="29" t="n"/>
+      <c r="N52" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B01HOYD69Q?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O52" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P52" s="31" t="n"/>
-      <c r="Q52" s="29" t="n"/>
-      <c r="R52" s="32" t="n"/>
-      <c r="S52" s="28" t="n"/>
+      <c r="Q52" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R52" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S52" s="28" t="inlineStr">
+        <is>
+          <t>Catalog slug: hedgehog-food-exotic-nutrition-complete.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="41" t="inlineStr">
@@ -3741,22 +4501,54 @@
       <c r="H53" s="28" t="inlineStr"/>
       <c r="I53" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J53" s="28" t="n"/>
-      <c r="K53" s="29" t="n"/>
-      <c r="L53" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J53" s="28" t="inlineStr">
+        <is>
+          <t>API Aquarium Salt, 33 oz</t>
+        </is>
+      </c>
+      <c r="K53" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L53" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0010P82UO</t>
+        </is>
+      </c>
       <c r="M53" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L53)),MID(L53,SEARCH("/dp/",L53)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N53" s="28" t="n"/>
-      <c r="O53" s="29" t="n"/>
+      <c r="N53" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0010P82UO?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O53" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P53" s="31" t="n"/>
-      <c r="Q53" s="29" t="n"/>
-      <c r="R53" s="32" t="n"/>
-      <c r="S53" s="28" t="n"/>
+      <c r="Q53" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R53" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S53" s="28" t="inlineStr">
+        <is>
+          <t>Catalog slug: aquarium-salt-api-33oz.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="41" t="inlineStr">
@@ -3795,22 +4587,54 @@
       <c r="H54" s="28" t="inlineStr"/>
       <c r="I54" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J54" s="28" t="n"/>
-      <c r="K54" s="29" t="n"/>
-      <c r="L54" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J54" s="28" t="inlineStr">
+        <is>
+          <t>Kaytee Pine Bedding, 19.7 L</t>
+        </is>
+      </c>
+      <c r="K54" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L54" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B000LNQNHK</t>
+        </is>
+      </c>
       <c r="M54" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L54)),MID(L54,SEARCH("/dp/",L54)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N54" s="28" t="n"/>
-      <c r="O54" s="29" t="n"/>
+      <c r="N54" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B000LNQNHK?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O54" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P54" s="31" t="n"/>
-      <c r="Q54" s="29" t="n"/>
-      <c r="R54" s="32" t="n"/>
-      <c r="S54" s="28" t="n"/>
+      <c r="Q54" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R54" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S54" s="28" t="inlineStr">
+        <is>
+          <t>Catalog slug: bedding-kaytee-pine-19l.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="42" t="inlineStr">

</xml_diff>

<commit_message>
Add 47 more sourced products to the gear catalog and link 8 cost guide rows
Tier 4 of NEEDS_PRODUCT.xlsx: aquarium lids and maintenance gear, reptile
lids, clips and substrates, and bird and small mammal gear. Weak or unfound
picks stay open in NEEDS_PRODUCT.md with search notes in the sheet. Photos
needed are listed per row as product-311 to product-357.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012EvHa8anGf58M3dpjKW87b
</commit_message>
<xml_diff>
--- a/NEEDS_PRODUCT.xlsx
+++ b/NEEDS_PRODUCT.xlsx
@@ -4713,22 +4713,55 @@
       <c r="H55" s="28" t="inlineStr"/>
       <c r="I55" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J55" s="28" t="n"/>
-      <c r="K55" s="29" t="n"/>
-      <c r="L55" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J55" s="28" t="inlineStr">
+        <is>
+          <t>Aqueon Versa Top Hinged Glass Lid, 30 in</t>
+        </is>
+      </c>
+      <c r="K55" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L55" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0002AS802</t>
+        </is>
+      </c>
       <c r="M55" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L55)),MID(L55,SEARCH("/dp/",L55)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N55" s="28" t="n"/>
-      <c r="O55" s="29" t="n"/>
+      <c r="N55" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0002AS802?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O55" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P55" s="31" t="n"/>
-      <c r="Q55" s="29" t="n"/>
-      <c r="R55" s="32" t="n"/>
-      <c r="S55" s="28" t="n"/>
+      <c r="Q55" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R55" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S55" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-311.jpg = Aqueon Versa Top Hinged Glass Lid, 30 in (amazon.com/dp/B0002AS802)
+Catalog slug: glass-lid-aqueon-versa-top-30in.</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="42" t="inlineStr">
@@ -4767,22 +4800,55 @@
       <c r="H56" s="28" t="inlineStr"/>
       <c r="I56" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J56" s="28" t="n"/>
-      <c r="K56" s="29" t="n"/>
-      <c r="L56" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J56" s="28" t="inlineStr">
+        <is>
+          <t>Arcadia PureSun Compact Bird Lighting Kit</t>
+        </is>
+      </c>
+      <c r="K56" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L56" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B009SAZW10</t>
+        </is>
+      </c>
       <c r="M56" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L56)),MID(L56,SEARCH("/dp/",L56)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N56" s="28" t="n"/>
-      <c r="O56" s="29" t="n"/>
+      <c r="N56" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B009SAZW10?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O56" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P56" s="31" t="n"/>
-      <c r="Q56" s="29" t="n"/>
-      <c r="R56" s="32" t="n"/>
-      <c r="S56" s="28" t="n"/>
+      <c r="Q56" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R56" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S56" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-345.jpg = Arcadia PureSun Compact Bird Lighting Kit (amazon.com/dp/B009SAZW10)
+Catalog slug: uvb-arcadia-puresun-compact-bird-kit.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="42" t="inlineStr">
@@ -4836,7 +4902,11 @@
       <c r="P57" s="31" t="n"/>
       <c r="Q57" s="29" t="n"/>
       <c r="R57" s="32" t="n"/>
-      <c r="S57" s="28" t="n"/>
+      <c r="S57" s="28" t="inlineStr">
+        <is>
+          <t>Searched 2026-09-28, not added (weak or no match): Arcadia Jungle Dawn 34 in, 51W (B07XF7F86J), just under 36 in and about 6200K; or Bio Dude Solar Grow 36 in (B0DP3M61DP), Kelvin unconfirmed.</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="42" t="inlineStr">
@@ -4879,22 +4949,55 @@
       </c>
       <c r="I58" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J58" s="28" t="n"/>
-      <c r="K58" s="29" t="n"/>
-      <c r="L58" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J58" s="28" t="inlineStr">
+        <is>
+          <t>The Bio Dude Glow and Grow LED, 16 in</t>
+        </is>
+      </c>
+      <c r="K58" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L58" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B099NRFK6T</t>
+        </is>
+      </c>
       <c r="M58" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L58)),MID(L58,SEARCH("/dp/",L58)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N58" s="28" t="n"/>
-      <c r="O58" s="29" t="n"/>
+      <c r="N58" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B099NRFK6T?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O58" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P58" s="31" t="n"/>
-      <c r="Q58" s="29" t="n"/>
-      <c r="R58" s="32" t="n"/>
-      <c r="S58" s="28" t="n"/>
+      <c r="Q58" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R58" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S58" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-330.jpg = The Bio Dude Glow and Grow LED, 16 in (amazon.com/dp/B099NRFK6T)
+Catalog slug: grow-light-bio-dude-glow-grow-16in.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="42" t="inlineStr">
@@ -4937,22 +5040,55 @@
       </c>
       <c r="I59" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J59" s="28" t="n"/>
-      <c r="K59" s="29" t="n"/>
-      <c r="L59" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J59" s="28" t="inlineStr">
+        <is>
+          <t>Aqueon Versa Top Hinged Glass Lid, 20 in</t>
+        </is>
+      </c>
+      <c r="K59" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L59" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0002AS7ZI</t>
+        </is>
+      </c>
       <c r="M59" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L59)),MID(L59,SEARCH("/dp/",L59)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N59" s="28" t="n"/>
-      <c r="O59" s="29" t="n"/>
+      <c r="N59" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0002AS7ZI?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O59" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P59" s="31" t="n"/>
-      <c r="Q59" s="29" t="n"/>
-      <c r="R59" s="32" t="n"/>
-      <c r="S59" s="28" t="n"/>
+      <c r="Q59" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R59" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S59" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-312.jpg = Aqueon Versa Top Hinged Glass Lid, 20 in (amazon.com/dp/B0002AS7ZI)
+Catalog slug: glass-lid-aqueon-versa-top-20in.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="42" t="inlineStr">
@@ -4991,22 +5127,55 @@
       <c r="H60" s="28" t="inlineStr"/>
       <c r="I60" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J60" s="28" t="n"/>
-      <c r="K60" s="29" t="n"/>
-      <c r="L60" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J60" s="28" t="inlineStr">
+        <is>
+          <t>Daltile Natural Slate Tile, 12x12 in, 6 Pack</t>
+        </is>
+      </c>
+      <c r="K60" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L60" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0CKZWLWT3</t>
+        </is>
+      </c>
       <c r="M60" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L60)),MID(L60,SEARCH("/dp/",L60)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N60" s="28" t="n"/>
-      <c r="O60" s="29" t="n"/>
+      <c r="N60" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0CKZWLWT3?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O60" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P60" s="31" t="n"/>
-      <c r="Q60" s="29" t="n"/>
-      <c r="R60" s="32" t="n"/>
-      <c r="S60" s="28" t="n"/>
+      <c r="Q60" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R60" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S60" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-331.jpg = Daltile Natural Slate Tile, 12x12 in, 6 Pack (amazon.com/dp/B0CKZWLWT3)
+Catalog slug: slate-tile-daltile-12x12-6pack.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="42" t="inlineStr">
@@ -5045,22 +5214,55 @@
       <c r="H61" s="28" t="inlineStr"/>
       <c r="I61" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J61" s="28" t="n"/>
-      <c r="K61" s="29" t="n"/>
-      <c r="L61" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J61" s="28" t="inlineStr">
+        <is>
+          <t>AquaTop 5 in Fine Mesh Aquarium Net</t>
+        </is>
+      </c>
+      <c r="K61" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L61" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B01LVYOCKO</t>
+        </is>
+      </c>
       <c r="M61" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L61)),MID(L61,SEARCH("/dp/",L61)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N61" s="28" t="n"/>
-      <c r="O61" s="29" t="n"/>
+      <c r="N61" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B01LVYOCKO?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O61" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P61" s="31" t="n"/>
-      <c r="Q61" s="29" t="n"/>
-      <c r="R61" s="32" t="n"/>
-      <c r="S61" s="28" t="n"/>
+      <c r="Q61" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R61" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S61" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-323.jpg = AquaTop 5 in Fine Mesh Aquarium Net (amazon.com/dp/B01LVYOCKO); product-324.jpg = Aquascape Heavy Duty Pond Net, 36 to 69 in Extendable (amazon.com/dp/B0039G5HCI)
+Catalog slug: net-aquatop-5in-fine-mesh, net-aquascape-pond-extendable. Also added: Aquascape Heavy Duty Pond Net, 36 to 69 in Extendable (https://www.amazon.com/dp/B0039G5HCI).</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="42" t="inlineStr">
@@ -5099,22 +5301,55 @@
       <c r="H62" s="28" t="inlineStr"/>
       <c r="I62" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J62" s="28" t="n"/>
-      <c r="K62" s="29" t="n"/>
-      <c r="L62" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J62" s="28" t="inlineStr">
+        <is>
+          <t>GuineaDad Original Fleece Cage Liner</t>
+        </is>
+      </c>
+      <c r="K62" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L62" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B076D27KNB</t>
+        </is>
+      </c>
       <c r="M62" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L62)),MID(L62,SEARCH("/dp/",L62)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N62" s="28" t="n"/>
-      <c r="O62" s="29" t="n"/>
+      <c r="N62" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B076D27KNB?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O62" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P62" s="31" t="n"/>
-      <c r="Q62" s="29" t="n"/>
-      <c r="R62" s="32" t="n"/>
-      <c r="S62" s="28" t="n"/>
+      <c r="Q62" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R62" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S62" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-346.jpg = GuineaDad Original Fleece Cage Liner (amazon.com/dp/B076D27KNB)
+Catalog slug: fleece-liner-guineadad-original.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="42" t="inlineStr">
@@ -5153,22 +5388,55 @@
       <c r="H63" s="28" t="inlineStr"/>
       <c r="I63" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J63" s="28" t="n"/>
-      <c r="K63" s="29" t="n"/>
-      <c r="L63" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J63" s="28" t="inlineStr">
+        <is>
+          <t>CaribSea Tahitian Moon Black Aquarium Sand, 20 lb</t>
+        </is>
+      </c>
+      <c r="K63" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L63" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B007R55QUU</t>
+        </is>
+      </c>
       <c r="M63" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L63)),MID(L63,SEARCH("/dp/",L63)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N63" s="28" t="n"/>
-      <c r="O63" s="29" t="n"/>
+      <c r="N63" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B007R55QUU?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O63" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P63" s="31" t="n"/>
-      <c r="Q63" s="29" t="n"/>
-      <c r="R63" s="32" t="n"/>
-      <c r="S63" s="28" t="n"/>
+      <c r="Q63" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R63" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S63" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-317.jpg = CaribSea Tahitian Moon Black Aquarium Sand, 20 lb (amazon.com/dp/B007R55QUU)
+Catalog slug: sand-caribsea-tahitian-moon-20lb.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="42" t="inlineStr">
@@ -5207,22 +5475,55 @@
       <c r="H64" s="28" t="inlineStr"/>
       <c r="I64" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J64" s="28" t="n"/>
-      <c r="K64" s="29" t="n"/>
-      <c r="L64" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J64" s="28" t="inlineStr">
+        <is>
+          <t>Python Pro-Clean Gravel Washer and Siphon, Large, with Squeeze Bulb</t>
+        </is>
+      </c>
+      <c r="K64" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L64" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B00BDPFX62</t>
+        </is>
+      </c>
       <c r="M64" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L64)),MID(L64,SEARCH("/dp/",L64)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N64" s="28" t="n"/>
-      <c r="O64" s="29" t="n"/>
+      <c r="N64" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B00BDPFX62?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O64" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P64" s="31" t="n"/>
-      <c r="Q64" s="29" t="n"/>
-      <c r="R64" s="32" t="n"/>
-      <c r="S64" s="28" t="n"/>
+      <c r="Q64" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R64" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S64" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-318.jpg = Python Pro-Clean Gravel Washer and Siphon, Large, with Squeeze Bulb (amazon.com/dp/B00BDPFX62)
+Catalog slug: gravel-vac-python-pro-clean-large.</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="42" t="inlineStr">
@@ -5261,22 +5562,55 @@
       <c r="H65" s="28" t="inlineStr"/>
       <c r="I65" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J65" s="28" t="n"/>
-      <c r="K65" s="29" t="n"/>
-      <c r="L65" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J65" s="28" t="inlineStr">
+        <is>
+          <t>Tetra 29 Gallon Glass Aquarium, Tank Only</t>
+        </is>
+      </c>
+      <c r="K65" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L65" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B08BJ9FQY7</t>
+        </is>
+      </c>
       <c r="M65" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L65)),MID(L65,SEARCH("/dp/",L65)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N65" s="28" t="n"/>
-      <c r="O65" s="29" t="n"/>
+      <c r="N65" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B08BJ9FQY7?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O65" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P65" s="31" t="n"/>
-      <c r="Q65" s="29" t="n"/>
-      <c r="R65" s="32" t="n"/>
-      <c r="S65" s="28" t="n"/>
+      <c r="Q65" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R65" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S65" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-315.jpg = Tetra 29 Gallon Glass Aquarium, Tank Only (amazon.com/dp/B08BJ9FQY7)
+Catalog slug: tank-tetra-29-gallon.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="42" t="inlineStr">
@@ -5315,22 +5649,55 @@
       <c r="H66" s="28" t="inlineStr"/>
       <c r="I66" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J66" s="28" t="n"/>
-      <c r="K66" s="29" t="n"/>
-      <c r="L66" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J66" s="28" t="inlineStr">
+        <is>
+          <t>AQUANEAT Pre-Filter Sponge, 6 Pack (0.8 in intake)</t>
+        </is>
+      </c>
+      <c r="K66" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L66" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0B5KW55YX</t>
+        </is>
+      </c>
       <c r="M66" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L66)),MID(L66,SEARCH("/dp/",L66)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N66" s="28" t="n"/>
-      <c r="O66" s="29" t="n"/>
+      <c r="N66" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0B5KW55YX?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O66" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P66" s="31" t="n"/>
-      <c r="Q66" s="29" t="n"/>
-      <c r="R66" s="32" t="n"/>
-      <c r="S66" s="28" t="n"/>
+      <c r="Q66" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R66" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S66" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-320.jpg = AQUANEAT Pre-Filter Sponge, 6 Pack (0.8 in intake) (amazon.com/dp/B0B5KW55YX)
+Catalog slug: prefilter-sponge-aquaneat-6pack.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="42" t="inlineStr">
@@ -5369,22 +5736,55 @@
       <c r="H67" s="28" t="inlineStr"/>
       <c r="I67" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J67" s="28" t="n"/>
-      <c r="K67" s="29" t="n"/>
-      <c r="L67" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J67" s="28" t="inlineStr">
+        <is>
+          <t>Prevue Large Parrot Playstand with Wheels</t>
+        </is>
+      </c>
+      <c r="K67" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L67" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B000S13JIG</t>
+        </is>
+      </c>
       <c r="M67" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L67)),MID(L67,SEARCH("/dp/",L67)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N67" s="28" t="n"/>
-      <c r="O67" s="29" t="n"/>
+      <c r="N67" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B000S13JIG?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O67" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P67" s="31" t="n"/>
-      <c r="Q67" s="29" t="n"/>
-      <c r="R67" s="32" t="n"/>
-      <c r="S67" s="28" t="n"/>
+      <c r="Q67" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R67" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S67" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-347.jpg = Prevue Large Parrot Playstand with Wheels (amazon.com/dp/B000S13JIG)
+Catalog slug: play-stand-prevue-large-parrot.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="42" t="inlineStr">
@@ -5423,22 +5823,55 @@
       <c r="H68" s="28" t="inlineStr"/>
       <c r="I68" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J68" s="28" t="n"/>
-      <c r="K68" s="29" t="n"/>
-      <c r="L68" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J68" s="28" t="inlineStr">
+        <is>
+          <t>Dubia Farms 32 oz Deli Cups with Vented Lids, 10 Pack</t>
+        </is>
+      </c>
+      <c r="K68" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L68" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0FXT3SPDZ</t>
+        </is>
+      </c>
       <c r="M68" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L68)),MID(L68,SEARCH("/dp/",L68)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N68" s="28" t="n"/>
-      <c r="O68" s="29" t="n"/>
+      <c r="N68" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0FXT3SPDZ?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O68" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P68" s="31" t="n"/>
-      <c r="Q68" s="29" t="n"/>
-      <c r="R68" s="32" t="n"/>
-      <c r="S68" s="28" t="n"/>
+      <c r="Q68" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R68" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S68" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-332.jpg = Dubia Farms 32 oz Deli Cups with Vented Lids, 10 Pack (amazon.com/dp/B0FXT3SPDZ)
+Catalog slug: deli-cups-dubia-farms-32oz-vented.</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="42" t="inlineStr">
@@ -5492,7 +5925,11 @@
       <c r="P69" s="31" t="n"/>
       <c r="Q69" s="29" t="n"/>
       <c r="R69" s="32" t="n"/>
-      <c r="S69" s="28" t="n"/>
+      <c r="S69" s="28" t="inlineStr">
+        <is>
+          <t>Searched 2026-09-28, not added (weak or no match): Small sellers only: 10 piece kiln dried pine ledges (B0B79XPGYM); ledges with hardware (B075SJ3L2Q).</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="42" t="inlineStr">
@@ -5531,22 +5968,55 @@
       <c r="H70" s="28" t="inlineStr"/>
       <c r="I70" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J70" s="28" t="n"/>
-      <c r="K70" s="29" t="n"/>
-      <c r="L70" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J70" s="28" t="inlineStr">
+        <is>
+          <t>Zoo Med Eco Earth Coconut Chips, Brick</t>
+        </is>
+      </c>
+      <c r="K70" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L70" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0CKY4YGZ3</t>
+        </is>
+      </c>
       <c r="M70" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L70)),MID(L70,SEARCH("/dp/",L70)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N70" s="28" t="n"/>
-      <c r="O70" s="29" t="n"/>
+      <c r="N70" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0CKY4YGZ3?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O70" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P70" s="31" t="n"/>
-      <c r="Q70" s="29" t="n"/>
-      <c r="R70" s="32" t="n"/>
-      <c r="S70" s="28" t="n"/>
+      <c r="Q70" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R70" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S70" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-333.jpg = Zoo Med Eco Earth Coconut Chips, Brick (amazon.com/dp/B0CKY4YGZ3)
+Catalog slug: substrate-zoo-med-eco-earth-coconut-chips.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="42" t="inlineStr">
@@ -5585,22 +6055,55 @@
       <c r="H71" s="28" t="inlineStr"/>
       <c r="I71" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J71" s="28" t="n"/>
-      <c r="K71" s="29" t="n"/>
-      <c r="L71" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J71" s="28" t="inlineStr">
+        <is>
+          <t>Aqueon Versa Top Hinged Glass Lid, 48 in</t>
+        </is>
+      </c>
+      <c r="K71" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L71" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0002AS8D4</t>
+        </is>
+      </c>
       <c r="M71" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L71)),MID(L71,SEARCH("/dp/",L71)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N71" s="28" t="n"/>
-      <c r="O71" s="29" t="n"/>
+      <c r="N71" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0002AS8D4?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O71" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P71" s="31" t="n"/>
-      <c r="Q71" s="29" t="n"/>
-      <c r="R71" s="32" t="n"/>
-      <c r="S71" s="28" t="n"/>
+      <c r="Q71" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R71" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S71" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-313.jpg = Aqueon Versa Top Hinged Glass Lid, 48 in (amazon.com/dp/B0002AS8D4)
+Catalog slug: glass-lid-aqueon-versa-top-48in.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="42" t="inlineStr">
@@ -5639,22 +6142,55 @@
       <c r="H72" s="28" t="inlineStr"/>
       <c r="I72" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J72" s="28" t="n"/>
-      <c r="K72" s="29" t="n"/>
-      <c r="L72" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J72" s="28" t="inlineStr">
+        <is>
+          <t>Zilla Fresh Air Screen Cover, 36x18 in</t>
+        </is>
+      </c>
+      <c r="K72" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L72" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B000QFQ30K</t>
+        </is>
+      </c>
       <c r="M72" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L72)),MID(L72,SEARCH("/dp/",L72)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N72" s="28" t="n"/>
-      <c r="O72" s="29" t="n"/>
+      <c r="N72" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B000QFQ30K?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O72" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P72" s="31" t="n"/>
-      <c r="Q72" s="29" t="n"/>
-      <c r="R72" s="32" t="n"/>
-      <c r="S72" s="28" t="n"/>
+      <c r="Q72" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R72" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S72" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-334.jpg = Zilla Fresh Air Screen Cover, 36x18 in (amazon.com/dp/B000QFQ30K)
+Catalog slug: screen-lid-zilla-36x18.</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="42" t="inlineStr">
@@ -5693,22 +6229,55 @@
       <c r="H73" s="28" t="inlineStr"/>
       <c r="I73" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J73" s="28" t="n"/>
-      <c r="K73" s="29" t="n"/>
-      <c r="L73" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J73" s="28" t="inlineStr">
+        <is>
+          <t>Penn-Plax Standard Airline Tubing, 3/16 in, 25 ft</t>
+        </is>
+      </c>
+      <c r="K73" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L73" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0002563MW</t>
+        </is>
+      </c>
       <c r="M73" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L73)),MID(L73,SEARCH("/dp/",L73)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N73" s="28" t="n"/>
-      <c r="O73" s="29" t="n"/>
+      <c r="N73" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0002563MW?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O73" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P73" s="31" t="n"/>
-      <c r="Q73" s="29" t="n"/>
-      <c r="R73" s="32" t="n"/>
-      <c r="S73" s="28" t="n"/>
+      <c r="Q73" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R73" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S73" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-321.jpg = Penn-Plax Standard Airline Tubing, 3/16 in, 25 ft (amazon.com/dp/B0002563MW)
+Catalog slug: airline-penn-plax-25ft.</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="42" t="inlineStr">
@@ -5747,22 +6316,55 @@
       <c r="H74" s="28" t="inlineStr"/>
       <c r="I74" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J74" s="28" t="n"/>
-      <c r="K74" s="29" t="n"/>
-      <c r="L74" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J74" s="28" t="inlineStr">
+        <is>
+          <t>hygger Mini Aquarium Air Pump Kit, 2 to 20 Gallon</t>
+        </is>
+      </c>
+      <c r="K74" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L74" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B07XP4TMVW</t>
+        </is>
+      </c>
       <c r="M74" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L74)),MID(L74,SEARCH("/dp/",L74)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N74" s="28" t="n"/>
-      <c r="O74" s="29" t="n"/>
+      <c r="N74" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B07XP4TMVW?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O74" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P74" s="31" t="n"/>
-      <c r="Q74" s="29" t="n"/>
-      <c r="R74" s="32" t="n"/>
-      <c r="S74" s="28" t="n"/>
+      <c r="Q74" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R74" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S74" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-322.jpg = hygger Mini Aquarium Air Pump Kit, 2 to 20 Gallon (amazon.com/dp/B07XP4TMVW)
+Catalog slug: air-pump-hygger-mini-2-20gal.</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="42" t="inlineStr">
@@ -5805,22 +6407,55 @@
       </c>
       <c r="I75" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J75" s="28" t="n"/>
-      <c r="K75" s="29" t="n"/>
-      <c r="L75" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J75" s="28" t="inlineStr">
+        <is>
+          <t>Python No Spill Clean and Fill, 25 ft</t>
+        </is>
+      </c>
+      <c r="K75" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L75" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B000255NXC</t>
+        </is>
+      </c>
       <c r="M75" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L75)),MID(L75,SEARCH("/dp/",L75)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N75" s="28" t="n"/>
-      <c r="O75" s="29" t="n"/>
+      <c r="N75" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B000255NXC?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O75" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P75" s="31" t="n"/>
-      <c r="Q75" s="29" t="n"/>
-      <c r="R75" s="32" t="n"/>
-      <c r="S75" s="28" t="n"/>
+      <c r="Q75" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R75" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S75" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-319.jpg = Python No Spill Clean and Fill, 25 ft (amazon.com/dp/B000255NXC)
+Catalog slug: water-change-python-no-spill-25ft.</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="42" t="inlineStr">
@@ -5859,22 +6494,55 @@
       <c r="H76" s="28" t="inlineStr"/>
       <c r="I76" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J76" s="28" t="n"/>
-      <c r="K76" s="29" t="n"/>
-      <c r="L76" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J76" s="28" t="inlineStr">
+        <is>
+          <t>Aqueon Aquarium Silicone Sealant, Clear, 3 oz</t>
+        </is>
+      </c>
+      <c r="K76" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L76" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0002ASD2K</t>
+        </is>
+      </c>
       <c r="M76" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L76)),MID(L76,SEARCH("/dp/",L76)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N76" s="28" t="n"/>
-      <c r="O76" s="29" t="n"/>
+      <c r="N76" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0002ASD2K?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O76" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P76" s="31" t="n"/>
-      <c r="Q76" s="29" t="n"/>
-      <c r="R76" s="32" t="n"/>
-      <c r="S76" s="28" t="n"/>
+      <c r="Q76" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R76" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S76" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-325.jpg = Aqueon Aquarium Silicone Sealant, Clear, 3 oz (amazon.com/dp/B0002ASD2K)
+Catalog slug: silicone-aqueon-aquarium-sealant.</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="42" t="inlineStr">
@@ -5928,7 +6596,11 @@
       <c r="P77" s="31" t="n"/>
       <c r="Q77" s="29" t="n"/>
       <c r="R77" s="32" t="n"/>
-      <c r="S77" s="28" t="n"/>
+      <c r="S77" s="28" t="inlineStr">
+        <is>
+          <t>Searched 2026-09-28, not added (weak or no match): House Naturals food grade 3 pack with lids (B093GPG7M5), unknown brand.</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="42" t="inlineStr">
@@ -5967,22 +6639,55 @@
       <c r="H78" s="28" t="inlineStr"/>
       <c r="I78" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J78" s="28" t="n"/>
-      <c r="K78" s="29" t="n"/>
-      <c r="L78" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J78" s="28" t="inlineStr">
+        <is>
+          <t>Kaytee Natural Wooden Hay Manger, Large</t>
+        </is>
+      </c>
+      <c r="K78" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L78" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B005FU4Z74</t>
+        </is>
+      </c>
       <c r="M78" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L78)),MID(L78,SEARCH("/dp/",L78)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N78" s="28" t="n"/>
-      <c r="O78" s="29" t="n"/>
+      <c r="N78" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B005FU4Z74?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O78" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P78" s="31" t="n"/>
-      <c r="Q78" s="29" t="n"/>
-      <c r="R78" s="32" t="n"/>
-      <c r="S78" s="28" t="n"/>
+      <c r="Q78" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R78" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S78" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-348.jpg = Kaytee Natural Wooden Hay Manger, Large (amazon.com/dp/B005FU4Z74)
+Catalog slug: hay-manger-kaytee-large.</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="42" t="inlineStr">
@@ -6040,7 +6745,11 @@
       <c r="P79" s="31" t="n"/>
       <c r="Q79" s="29" t="n"/>
       <c r="R79" s="32" t="n"/>
-      <c r="S79" s="28" t="n"/>
+      <c r="S79" s="28" t="inlineStr">
+        <is>
+          <t>Searched 2026-09-28, not added (weak or no match): SPORN black static cling 24x12 in (B007GCEDNU) is too small for 30 in and 48 in tanks; larger 79x17.5 in sheet is a little-known brand (B0GYWQ6C14).</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="42" t="inlineStr">
@@ -6079,22 +6788,55 @@
       <c r="H80" s="28" t="inlineStr"/>
       <c r="I80" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J80" s="28" t="n"/>
-      <c r="K80" s="29" t="n"/>
-      <c r="L80" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J80" s="28" t="inlineStr">
+        <is>
+          <t>Juvale 2 in Terracotta Pots, 10 Pack</t>
+        </is>
+      </c>
+      <c r="K80" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L80" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B071L2F7TT</t>
+        </is>
+      </c>
       <c r="M80" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L80)),MID(L80,SEARCH("/dp/",L80)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N80" s="28" t="n"/>
-      <c r="O80" s="29" t="n"/>
+      <c r="N80" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B071L2F7TT?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O80" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P80" s="31" t="n"/>
-      <c r="Q80" s="29" t="n"/>
-      <c r="R80" s="32" t="n"/>
-      <c r="S80" s="28" t="n"/>
+      <c r="Q80" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R80" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S80" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-338.jpg = Juvale 2 in Terracotta Pots, 10 Pack (amazon.com/dp/B071L2F7TT)
+Catalog slug: terracotta-pots-juvale-2in-10pack.</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="42" t="inlineStr">
@@ -6137,22 +6879,55 @@
       </c>
       <c r="I81" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J81" s="28" t="n"/>
-      <c r="K81" s="29" t="n"/>
-      <c r="L81" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J81" s="28" t="inlineStr">
+        <is>
+          <t>Kaytee Silent Spinner Wheel, 6.5 in</t>
+        </is>
+      </c>
+      <c r="K81" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L81" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B000A7DFUU</t>
+        </is>
+      </c>
       <c r="M81" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L81)),MID(L81,SEARCH("/dp/",L81)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N81" s="28" t="n"/>
-      <c r="O81" s="29" t="n"/>
+      <c r="N81" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B000A7DFUU?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O81" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P81" s="31" t="n"/>
-      <c r="Q81" s="29" t="n"/>
-      <c r="R81" s="32" t="n"/>
-      <c r="S81" s="28" t="n"/>
+      <c r="Q81" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R81" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S81" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-349.jpg = Kaytee Silent Spinner Wheel, 6.5 in (amazon.com/dp/B000A7DFUU)
+Catalog slug: wheel-kaytee-silent-spinner-6-5in.</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="42" t="inlineStr">
@@ -6191,22 +6966,55 @@
       <c r="H82" s="28" t="inlineStr"/>
       <c r="I82" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J82" s="28" t="n"/>
-      <c r="K82" s="29" t="n"/>
-      <c r="L82" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J82" s="28" t="inlineStr">
+        <is>
+          <t>Sugar Gliders USA Large Hanging Nesting Box</t>
+        </is>
+      </c>
+      <c r="K82" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L82" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B07FK7V7HC</t>
+        </is>
+      </c>
       <c r="M82" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L82)),MID(L82,SEARCH("/dp/",L82)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N82" s="28" t="n"/>
-      <c r="O82" s="29" t="n"/>
+      <c r="N82" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B07FK7V7HC?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O82" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P82" s="31" t="n"/>
-      <c r="Q82" s="29" t="n"/>
-      <c r="R82" s="32" t="n"/>
-      <c r="S82" s="28" t="n"/>
+      <c r="Q82" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R82" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S82" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-350.jpg = Sugar Gliders USA Large Hanging Nesting Box (amazon.com/dp/B07FK7V7HC)
+Catalog slug: nest-box-sugar-gliders-usa-large.</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="42" t="inlineStr">
@@ -6245,22 +7053,55 @@
       <c r="H83" s="28" t="inlineStr"/>
       <c r="I83" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J83" s="28" t="n"/>
-      <c r="K83" s="29" t="n"/>
-      <c r="L83" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J83" s="28" t="inlineStr">
+        <is>
+          <t>Zoo Med Excavator Clay Burrowing Substrate, 10 lb</t>
+        </is>
+      </c>
+      <c r="K83" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L83" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B000N5OM8S</t>
+        </is>
+      </c>
       <c r="M83" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L83)),MID(L83,SEARCH("/dp/",L83)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N83" s="28" t="n"/>
-      <c r="O83" s="29" t="n"/>
+      <c r="N83" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B000N5OM8S?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O83" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P83" s="31" t="n"/>
-      <c r="Q83" s="29" t="n"/>
-      <c r="R83" s="32" t="n"/>
-      <c r="S83" s="28" t="n"/>
+      <c r="Q83" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R83" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S83" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-339.jpg = Zoo Med Excavator Clay Burrowing Substrate, 10 lb (amazon.com/dp/B000N5OM8S)
+Catalog slug: substrate-zoo-med-excavator-clay-10lb.</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="42" t="inlineStr">
@@ -6299,22 +7140,55 @@
       <c r="H84" s="28" t="inlineStr"/>
       <c r="I84" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J84" s="28" t="n"/>
-      <c r="K84" s="29" t="n"/>
-      <c r="L84" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J84" s="28" t="inlineStr">
+        <is>
+          <t>Better-Gro Orchid Bark, 8 qt</t>
+        </is>
+      </c>
+      <c r="K84" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L84" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B005OK83CI</t>
+        </is>
+      </c>
       <c r="M84" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L84)),MID(L84,SEARCH("/dp/",L84)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N84" s="28" t="n"/>
-      <c r="O84" s="29" t="n"/>
+      <c r="N84" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B005OK83CI?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O84" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P84" s="31" t="n"/>
-      <c r="Q84" s="29" t="n"/>
-      <c r="R84" s="32" t="n"/>
-      <c r="S84" s="28" t="n"/>
+      <c r="Q84" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R84" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S84" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-340.jpg = Better-Gro Orchid Bark, 8 qt (amazon.com/dp/B005OK83CI)
+Catalog slug: orchid-bark-better-gro-8qt.</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="42" t="inlineStr">
@@ -6368,7 +7242,11 @@
       <c r="P85" s="31" t="n"/>
       <c r="Q85" s="29" t="n"/>
       <c r="R85" s="32" t="n"/>
-      <c r="S85" s="28" t="n"/>
+      <c r="S85" s="28" t="inlineStr">
+        <is>
+          <t>Searched 2026-09-28, not added (weak or no match): Only flake soil found: Critters Direct flake soil 5 lb (B0BVS5Z7HW), fermented hardwood, not chunks.</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="42" t="inlineStr">
@@ -6407,22 +7285,55 @@
       <c r="H86" s="28" t="inlineStr"/>
       <c r="I86" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J86" s="28" t="n"/>
-      <c r="K86" s="29" t="n"/>
-      <c r="L86" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J86" s="28" t="inlineStr">
+        <is>
+          <t>API GH and KH Test Kit</t>
+        </is>
+      </c>
+      <c r="K86" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L86" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B003SNCHMA</t>
+        </is>
+      </c>
       <c r="M86" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L86)),MID(L86,SEARCH("/dp/",L86)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N86" s="28" t="n"/>
-      <c r="O86" s="29" t="n"/>
+      <c r="N86" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B003SNCHMA?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O86" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P86" s="31" t="n"/>
-      <c r="Q86" s="29" t="n"/>
-      <c r="R86" s="32" t="n"/>
-      <c r="S86" s="28" t="n"/>
+      <c r="Q86" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R86" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S86" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-326.jpg = API GH and KH Test Kit (amazon.com/dp/B003SNCHMA)
+Catalog slug: test-kit-api-gh-kh.</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="42" t="inlineStr">
@@ -6461,22 +7372,55 @@
       <c r="H87" s="28" t="inlineStr"/>
       <c r="I87" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J87" s="28" t="n"/>
-      <c r="K87" s="29" t="n"/>
-      <c r="L87" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J87" s="28" t="inlineStr">
+        <is>
+          <t>Exo Terra Glass Terrarium, 12x12x18 in</t>
+        </is>
+      </c>
+      <c r="K87" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L87" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B000OQW98Q</t>
+        </is>
+      </c>
       <c r="M87" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L87)),MID(L87,SEARCH("/dp/",L87)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N87" s="28" t="n"/>
-      <c r="O87" s="29" t="n"/>
+      <c r="N87" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B000OQW98Q?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O87" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P87" s="31" t="n"/>
-      <c r="Q87" s="29" t="n"/>
-      <c r="R87" s="32" t="n"/>
-      <c r="S87" s="28" t="n"/>
+      <c r="Q87" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R87" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S87" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-337.jpg = Exo Terra Glass Terrarium, 12x12x18 in (amazon.com/dp/B000OQW98Q)
+Catalog slug: terrarium-exo-terra-12x12x18.</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="42" t="inlineStr">
@@ -6530,7 +7474,11 @@
       <c r="P88" s="31" t="n"/>
       <c r="Q88" s="29" t="n"/>
       <c r="R88" s="32" t="n"/>
-      <c r="S88" s="28" t="n"/>
+      <c r="S88" s="28" t="inlineStr">
+        <is>
+          <t>Searched 2026-09-28, not added (weak or no match): None found at about 20x10x10 in.</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="42" t="inlineStr">
@@ -6569,22 +7517,55 @@
       <c r="H89" s="28" t="inlineStr"/>
       <c r="I89" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J89" s="28" t="n"/>
-      <c r="K89" s="29" t="n"/>
-      <c r="L89" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J89" s="28" t="inlineStr">
+        <is>
+          <t>Aquatic Fundamentals 55 Gallon Upright Aquarium Stand</t>
+        </is>
+      </c>
+      <c r="K89" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L89" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B07P9W4HRW</t>
+        </is>
+      </c>
       <c r="M89" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L89)),MID(L89,SEARCH("/dp/",L89)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N89" s="28" t="n"/>
-      <c r="O89" s="29" t="n"/>
+      <c r="N89" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B07P9W4HRW?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O89" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P89" s="31" t="n"/>
-      <c r="Q89" s="29" t="n"/>
-      <c r="R89" s="32" t="n"/>
-      <c r="S89" s="28" t="n"/>
+      <c r="Q89" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R89" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S89" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-316.jpg = Aquatic Fundamentals 55 Gallon Upright Aquarium Stand (amazon.com/dp/B07P9W4HRW)
+Catalog slug: stand-aquatic-fundamentals-55.</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="42" t="inlineStr">
@@ -6623,22 +7604,55 @@
       <c r="H90" s="28" t="inlineStr"/>
       <c r="I90" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J90" s="28" t="n"/>
-      <c r="K90" s="29" t="n"/>
-      <c r="L90" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J90" s="28" t="inlineStr">
+        <is>
+          <t>Glass Canopy Set for 75 to 110 Gallon Tanks, 48x18 in</t>
+        </is>
+      </c>
+      <c r="K90" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L90" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B01N6MYOHS</t>
+        </is>
+      </c>
       <c r="M90" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L90)),MID(L90,SEARCH("/dp/",L90)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N90" s="28" t="n"/>
-      <c r="O90" s="29" t="n"/>
+      <c r="N90" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B01N6MYOHS?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O90" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P90" s="31" t="n"/>
-      <c r="Q90" s="29" t="n"/>
-      <c r="R90" s="32" t="n"/>
-      <c r="S90" s="28" t="n"/>
+      <c r="Q90" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R90" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S90" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-314.jpg = Glass Canopy Set for 75 to 110 Gallon Tanks, 48x18 in (amazon.com/dp/B01N6MYOHS)
+Catalog slug: glass-lid-48x18-center-brace.</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="42" t="inlineStr">
@@ -6677,22 +7691,55 @@
       <c r="H91" s="28" t="inlineStr"/>
       <c r="I91" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J91" s="28" t="n"/>
-      <c r="K91" s="29" t="n"/>
-      <c r="L91" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J91" s="28" t="inlineStr">
+        <is>
+          <t>Zilla Fresh Air Screen Cover, 20x10 in</t>
+        </is>
+      </c>
+      <c r="K91" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L91" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B000QFOGAE</t>
+        </is>
+      </c>
       <c r="M91" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L91)),MID(L91,SEARCH("/dp/",L91)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N91" s="28" t="n"/>
-      <c r="O91" s="29" t="n"/>
+      <c r="N91" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B000QFOGAE?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O91" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P91" s="31" t="n"/>
-      <c r="Q91" s="29" t="n"/>
-      <c r="R91" s="32" t="n"/>
-      <c r="S91" s="28" t="n"/>
+      <c r="Q91" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R91" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S91" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-335.jpg = Zilla Fresh Air Screen Cover, 20x10 in (amazon.com/dp/B000QFOGAE)
+Catalog slug: screen-lid-zilla-20x10.</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="42" t="inlineStr">
@@ -6746,7 +7793,11 @@
       <c r="P92" s="31" t="n"/>
       <c r="Q92" s="29" t="n"/>
       <c r="R92" s="32" t="n"/>
-      <c r="S92" s="28" t="n"/>
+      <c r="S92" s="28" t="inlineStr">
+        <is>
+          <t>Searched 2026-09-28, not added (weak or no match): Prevue Hendryx travel cage 20x12x16 (B005U72PLU), a travel cage and small for a grey.</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="42" t="inlineStr">
@@ -6785,22 +7836,55 @@
       <c r="H93" s="28" t="inlineStr"/>
       <c r="I93" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J93" s="28" t="n"/>
-      <c r="K93" s="29" t="n"/>
-      <c r="L93" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J93" s="28" t="inlineStr">
+        <is>
+          <t>Zilla Fresh Air Locking Screen Clips, 2 Pack</t>
+        </is>
+      </c>
+      <c r="K93" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L93" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B005KPLZN6</t>
+        </is>
+      </c>
       <c r="M93" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L93)),MID(L93,SEARCH("/dp/",L93)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N93" s="28" t="n"/>
-      <c r="O93" s="29" t="n"/>
+      <c r="N93" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B005KPLZN6?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O93" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P93" s="31" t="n"/>
-      <c r="Q93" s="29" t="n"/>
-      <c r="R93" s="32" t="n"/>
-      <c r="S93" s="28" t="n"/>
+      <c r="Q93" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R93" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S93" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-336.jpg = Zilla Fresh Air Locking Screen Clips, 2 Pack (amazon.com/dp/B005KPLZN6)
+Catalog slug: lid-clips-zilla-locking.</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="42" t="inlineStr">
@@ -6858,7 +7942,11 @@
       <c r="P94" s="31" t="n"/>
       <c r="Q94" s="29" t="n"/>
       <c r="R94" s="32" t="n"/>
-      <c r="S94" s="28" t="n"/>
+      <c r="S94" s="28" t="inlineStr">
+        <is>
+          <t>Searched 2026-09-28, not added (weak or no match): Aquascape 91017 AquaSurge (B007BK6I5I), confirm on the listing it is the 2000 GPH model; or AquaSurge 3000, 3,196 GPH (B07TSQW9MJ). Also check whether the catalog TotalPond kit includes a pump.</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="42" t="inlineStr">
@@ -6897,22 +7985,55 @@
       <c r="H95" s="28" t="inlineStr"/>
       <c r="I95" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J95" s="28" t="n"/>
-      <c r="K95" s="29" t="n"/>
-      <c r="L95" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J95" s="28" t="inlineStr">
+        <is>
+          <t>Fluval U1 Underwater Filter</t>
+        </is>
+      </c>
+      <c r="K95" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L95" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0020K966M</t>
+        </is>
+      </c>
       <c r="M95" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L95)),MID(L95,SEARCH("/dp/",L95)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N95" s="28" t="n"/>
-      <c r="O95" s="29" t="n"/>
+      <c r="N95" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0020K966M?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O95" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P95" s="31" t="n"/>
-      <c r="Q95" s="29" t="n"/>
-      <c r="R95" s="32" t="n"/>
-      <c r="S95" s="28" t="n"/>
+      <c r="Q95" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R95" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S95" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-328.jpg = Fluval U1 Underwater Filter (amazon.com/dp/B0020K966M)
+Catalog slug: filter-fluval-u1-internal.</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="42" t="inlineStr">
@@ -6951,22 +8072,55 @@
       <c r="H96" s="28" t="inlineStr"/>
       <c r="I96" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J96" s="28" t="n"/>
-      <c r="K96" s="29" t="n"/>
-      <c r="L96" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J96" s="28" t="inlineStr">
+        <is>
+          <t>Lixit Glass Bird Water Bottles, 16 oz, 2 Pack</t>
+        </is>
+      </c>
+      <c r="K96" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L96" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B07J6GWKDT</t>
+        </is>
+      </c>
       <c r="M96" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L96)),MID(L96,SEARCH("/dp/",L96)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N96" s="28" t="n"/>
-      <c r="O96" s="29" t="n"/>
+      <c r="N96" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B07J6GWKDT?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O96" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P96" s="31" t="n"/>
-      <c r="Q96" s="29" t="n"/>
-      <c r="R96" s="32" t="n"/>
-      <c r="S96" s="28" t="n"/>
+      <c r="Q96" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R96" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S96" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-351.jpg = Lixit Glass Bird Water Bottles, 16 oz, 2 Pack (amazon.com/dp/B07J6GWKDT)
+Catalog slug: water-bottle-lixit-bird-glass-16oz.</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="42" t="inlineStr">
@@ -7020,7 +8174,11 @@
       <c r="P97" s="31" t="n"/>
       <c r="Q97" s="29" t="n"/>
       <c r="R97" s="32" t="n"/>
-      <c r="S97" s="28" t="n"/>
+      <c r="S97" s="28" t="inlineStr">
+        <is>
+          <t>Searched 2026-09-28, not added (weak or no match): Niteangel ceramic hideout (B0BGN5KWD6), 2.1 in entrance may be too small for degus.</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="42" t="inlineStr">
@@ -7074,7 +8232,11 @@
       <c r="P98" s="31" t="n"/>
       <c r="Q98" s="29" t="n"/>
       <c r="R98" s="32" t="n"/>
-      <c r="S98" s="28" t="n"/>
+      <c r="S98" s="28" t="inlineStr">
+        <is>
+          <t>Searched 2026-09-28, not added (weak or no match): None found. Nearest: Zoo Med ReptiBreeze 24x24 bottom tray (B0164R03RW), fits only that cage and is not a drainage tray.</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="42" t="inlineStr">
@@ -7113,22 +8275,55 @@
       <c r="H99" s="28" t="inlineStr"/>
       <c r="I99" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J99" s="28" t="n"/>
-      <c r="K99" s="29" t="n"/>
-      <c r="L99" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J99" s="28" t="inlineStr">
+        <is>
+          <t>Polly's Pastel Safety Perch, Medium</t>
+        </is>
+      </c>
+      <c r="K99" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L99" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0CZ4DNM6J</t>
+        </is>
+      </c>
       <c r="M99" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L99)),MID(L99,SEARCH("/dp/",L99)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N99" s="28" t="n"/>
-      <c r="O99" s="29" t="n"/>
+      <c r="N99" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0CZ4DNM6J?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O99" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P99" s="31" t="n"/>
-      <c r="Q99" s="29" t="n"/>
-      <c r="R99" s="32" t="n"/>
-      <c r="S99" s="28" t="n"/>
+      <c r="Q99" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R99" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S99" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-352.jpg = Polly's Pastel Safety Perch, Medium (amazon.com/dp/B0CZ4DNM6J)
+Catalog slug: perch-pollys-pastel-medium.</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="42" t="inlineStr">
@@ -7167,22 +8362,55 @@
       <c r="H100" s="28" t="inlineStr"/>
       <c r="I100" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J100" s="28" t="n"/>
-      <c r="K100" s="29" t="n"/>
-      <c r="L100" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J100" s="28" t="inlineStr">
+        <is>
+          <t>SunGrow Cord Protector Tubing, 20 ft</t>
+        </is>
+      </c>
+      <c r="K100" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L100" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B07CZ8LL35</t>
+        </is>
+      </c>
       <c r="M100" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L100)),MID(L100,SEARCH("/dp/",L100)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N100" s="28" t="n"/>
-      <c r="O100" s="29" t="n"/>
+      <c r="N100" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B07CZ8LL35?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O100" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P100" s="31" t="n"/>
-      <c r="Q100" s="29" t="n"/>
-      <c r="R100" s="32" t="n"/>
-      <c r="S100" s="28" t="n"/>
+      <c r="Q100" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R100" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S100" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-353.jpg = SunGrow Cord Protector Tubing, 20 ft (amazon.com/dp/B07CZ8LL35)
+Catalog slug: cord-protector-sungrow-20ft.</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="42" t="inlineStr">
@@ -7221,22 +8449,55 @@
       <c r="H101" s="28" t="inlineStr"/>
       <c r="I101" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J101" s="28" t="n"/>
-      <c r="K101" s="29" t="n"/>
-      <c r="L101" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J101" s="28" t="inlineStr">
+        <is>
+          <t>Josh's Frogs Egg Flats, 15 Count</t>
+        </is>
+      </c>
+      <c r="K101" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L101" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B08ZVRNH7C</t>
+        </is>
+      </c>
       <c r="M101" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L101)),MID(L101,SEARCH("/dp/",L101)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N101" s="28" t="n"/>
-      <c r="O101" s="29" t="n"/>
+      <c r="N101" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B08ZVRNH7C?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O101" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P101" s="31" t="n"/>
-      <c r="Q101" s="29" t="n"/>
-      <c r="R101" s="32" t="n"/>
-      <c r="S101" s="28" t="n"/>
+      <c r="Q101" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R101" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S101" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-341.jpg = Josh's Frogs Egg Flats, 15 Count (amazon.com/dp/B08ZVRNH7C)
+Catalog slug: egg-flats-joshs-frogs-15.</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="42" t="inlineStr">
@@ -7275,22 +8536,55 @@
       <c r="H102" s="28" t="inlineStr"/>
       <c r="I102" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J102" s="28" t="n"/>
-      <c r="K102" s="29" t="n"/>
-      <c r="L102" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J102" s="28" t="inlineStr">
+        <is>
+          <t>Planet Pleasures Shredders Zig Zag Palm Roll, 30 ft</t>
+        </is>
+      </c>
+      <c r="K102" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L102" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0002FP43Q</t>
+        </is>
+      </c>
       <c r="M102" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L102)),MID(L102,SEARCH("/dp/",L102)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N102" s="28" t="n"/>
-      <c r="O102" s="29" t="n"/>
+      <c r="N102" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0002FP43Q?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O102" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P102" s="31" t="n"/>
-      <c r="Q102" s="29" t="n"/>
-      <c r="R102" s="32" t="n"/>
-      <c r="S102" s="28" t="n"/>
+      <c r="Q102" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R102" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S102" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-354.jpg = Planet Pleasures Shredders Zig Zag Palm Roll, 30 ft (amazon.com/dp/B0002FP43Q)
+Catalog slug: shredder-planet-pleasures-zig-zag.</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="42" t="inlineStr">
@@ -7329,22 +8623,55 @@
       <c r="H103" s="28" t="inlineStr"/>
       <c r="I103" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J103" s="28" t="n"/>
-      <c r="K103" s="29" t="n"/>
-      <c r="L103" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J103" s="28" t="inlineStr">
+        <is>
+          <t>Sandbaggy Geotextile Pond Underlayment, 6 ft x 50 ft</t>
+        </is>
+      </c>
+      <c r="K103" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L103" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B09VC3C6B8</t>
+        </is>
+      </c>
       <c r="M103" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L103)),MID(L103,SEARCH("/dp/",L103)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N103" s="28" t="n"/>
-      <c r="O103" s="29" t="n"/>
+      <c r="N103" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B09VC3C6B8?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O103" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P103" s="31" t="n"/>
-      <c r="Q103" s="29" t="n"/>
-      <c r="R103" s="32" t="n"/>
-      <c r="S103" s="28" t="n"/>
+      <c r="Q103" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R103" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S103" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-329.jpg = Sandbaggy Geotextile Pond Underlayment, 6 ft x 50 ft (amazon.com/dp/B09VC3C6B8)
+Catalog slug: pond-underlayment-sandbaggy-6x50.</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="42" t="inlineStr">
@@ -7398,7 +8725,11 @@
       <c r="P104" s="31" t="n"/>
       <c r="Q104" s="29" t="n"/>
       <c r="R104" s="32" t="n"/>
-      <c r="S104" s="28" t="n"/>
+      <c r="S104" s="28" t="inlineStr">
+        <is>
+          <t>Searched 2026-09-28, not added (weak or no match): REPTIZOO resin slate stack (B0BX35CM35) is light for a monitor; INOSCIND slate basking platform 15.7x11.8 in (B0CZXS1Z57).</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="42" t="inlineStr">
@@ -7452,7 +8783,11 @@
       <c r="P105" s="31" t="n"/>
       <c r="Q105" s="29" t="n"/>
       <c r="R105" s="32" t="n"/>
-      <c r="S105" s="28" t="n"/>
+      <c r="S105" s="28" t="inlineStr">
+        <is>
+          <t>Searched 2026-09-28, not added (weak or no match): Generic only: DIYEAH stainless door clips 10 pack (B0G154L6N6); half moon lock (B0GHSR1RZ9).</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="42" t="inlineStr">
@@ -7506,7 +8841,11 @@
       <c r="P106" s="31" t="n"/>
       <c r="Q106" s="29" t="n"/>
       <c r="R106" s="32" t="n"/>
-      <c r="S106" s="28" t="n"/>
+      <c r="S106" s="28" t="inlineStr">
+        <is>
+          <t>Searched 2026-09-28, not added (weak or no match): None found as a standalone product.</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="42" t="inlineStr">
@@ -7545,22 +8884,55 @@
       <c r="H107" s="28" t="inlineStr"/>
       <c r="I107" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J107" s="28" t="n"/>
-      <c r="K107" s="29" t="n"/>
-      <c r="L107" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J107" s="28" t="inlineStr">
+        <is>
+          <t>Prevue Playpen Cover and Floor Mat, Small</t>
+        </is>
+      </c>
+      <c r="K107" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L107" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B000WMN38M</t>
+        </is>
+      </c>
       <c r="M107" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L107)),MID(L107,SEARCH("/dp/",L107)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N107" s="28" t="n"/>
-      <c r="O107" s="29" t="n"/>
+      <c r="N107" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B000WMN38M?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O107" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P107" s="31" t="n"/>
-      <c r="Q107" s="29" t="n"/>
-      <c r="R107" s="32" t="n"/>
-      <c r="S107" s="28" t="n"/>
+      <c r="Q107" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R107" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S107" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-355.jpg = Prevue Playpen Cover and Floor Mat, Small (amazon.com/dp/B000WMN38M); product-356.jpg = Xpose Safety Heavy Duty Poly Tarp, 6x8 ft, 10 mil (amazon.com/dp/B07GYZLYGL)
+Catalog slug: pen-mat-prevue-playpen-cover, tarp-xpose-6x8-10mil. Also added: Xpose Safety Heavy Duty Poly Tarp, 6x8 ft, 10 mil (https://www.amazon.com/dp/B07GYZLYGL).</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="42" t="inlineStr">
@@ -7599,22 +8971,55 @@
       <c r="H108" s="28" t="inlineStr"/>
       <c r="I108" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J108" s="28" t="n"/>
-      <c r="K108" s="29" t="n"/>
-      <c r="L108" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J108" s="28" t="inlineStr">
+        <is>
+          <t>Royal Imports Floral Water Tubes with Caps, 25 Pack</t>
+        </is>
+      </c>
+      <c r="K108" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L108" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B08W9ND27F</t>
+        </is>
+      </c>
       <c r="M108" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L108)),MID(L108,SEARCH("/dp/",L108)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N108" s="28" t="n"/>
-      <c r="O108" s="29" t="n"/>
+      <c r="N108" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B08W9ND27F?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O108" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P108" s="31" t="n"/>
-      <c r="Q108" s="29" t="n"/>
-      <c r="R108" s="32" t="n"/>
-      <c r="S108" s="28" t="n"/>
+      <c r="Q108" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R108" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S108" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-342.jpg = Royal Imports Floral Water Tubes with Caps, 25 Pack (amazon.com/dp/B08W9ND27F)
+Catalog slug: water-tubes-royal-imports-25pack.</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="42" t="inlineStr">
@@ -7668,7 +9073,11 @@
       <c r="P109" s="31" t="n"/>
       <c r="Q109" s="29" t="n"/>
       <c r="R109" s="32" t="n"/>
-      <c r="S109" s="28" t="n"/>
+      <c r="S109" s="28" t="inlineStr">
+        <is>
+          <t>Searched 2026-09-28, not added (weak or no match): FANTIAN 2-3 in river rock 5 lb (B0CHR45RG5), small brand; alt B0H2WMLM1M. Avoid polished rock, which can be wax coated.</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="42" t="inlineStr">
@@ -7707,22 +9116,55 @@
       <c r="H110" s="28" t="inlineStr"/>
       <c r="I110" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J110" s="28" t="n"/>
-      <c r="K110" s="29" t="n"/>
-      <c r="L110" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J110" s="28" t="inlineStr">
+        <is>
+          <t>HM Digital TDS-3 Handheld TDS Meter</t>
+        </is>
+      </c>
+      <c r="K110" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L110" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B000VTQM70</t>
+        </is>
+      </c>
       <c r="M110" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L110)),MID(L110,SEARCH("/dp/",L110)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N110" s="28" t="n"/>
-      <c r="O110" s="29" t="n"/>
+      <c r="N110" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B000VTQM70?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O110" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P110" s="31" t="n"/>
-      <c r="Q110" s="29" t="n"/>
-      <c r="R110" s="32" t="n"/>
-      <c r="S110" s="28" t="n"/>
+      <c r="Q110" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R110" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S110" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-327.jpg = HM Digital TDS-3 Handheld TDS Meter (amazon.com/dp/B000VTQM70)
+Catalog slug: tds-meter-hm-digital-tds3.</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="42" t="inlineStr">
@@ -7761,22 +9203,55 @@
       <c r="H111" s="28" t="inlineStr"/>
       <c r="I111" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J111" s="28" t="n"/>
-      <c r="K111" s="29" t="n"/>
-      <c r="L111" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J111" s="28" t="inlineStr">
+        <is>
+          <t>REScue One-Step Ready to Use Disinfectant Cleaner</t>
+        </is>
+      </c>
+      <c r="K111" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L111" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B01LY3JI7T</t>
+        </is>
+      </c>
       <c r="M111" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L111)),MID(L111,SEARCH("/dp/",L111)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N111" s="28" t="n"/>
-      <c r="O111" s="29" t="n"/>
+      <c r="N111" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B01LY3JI7T?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O111" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P111" s="31" t="n"/>
-      <c r="Q111" s="29" t="n"/>
-      <c r="R111" s="32" t="n"/>
-      <c r="S111" s="28" t="n"/>
+      <c r="Q111" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R111" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S111" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-357.jpg = REScue One-Step Ready to Use Disinfectant Cleaner (amazon.com/dp/B01LY3JI7T)
+Catalog slug: disinfectant-rescue-one-step-rtu.</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="42" t="inlineStr">
@@ -7830,7 +9305,11 @@
       <c r="P112" s="31" t="n"/>
       <c r="Q112" s="29" t="n"/>
       <c r="R112" s="32" t="n"/>
-      <c r="S112" s="28" t="n"/>
+      <c r="S112" s="28" t="inlineStr">
+        <is>
+          <t>Searched 2026-09-28, not added (weak or no match): Uniclife 64 GPH kit (B01EBXI7PG), small brand; or Tetra Whisper 60-100 gal, pump only (B004PB8SRM).</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="42" t="inlineStr">
@@ -7869,22 +9348,55 @@
       <c r="H113" s="28" t="inlineStr"/>
       <c r="I113" s="29" t="inlineStr">
         <is>
-          <t>To find</t>
-        </is>
-      </c>
-      <c r="J113" s="28" t="n"/>
-      <c r="K113" s="29" t="n"/>
-      <c r="L113" s="28" t="n"/>
+          <t>Added to catalog</t>
+        </is>
+      </c>
+      <c r="J113" s="28" t="inlineStr">
+        <is>
+          <t>Josh's Frogs LECA Expanded Clay Pebbles</t>
+        </is>
+      </c>
+      <c r="K113" s="29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="L113" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B00JJVBXHK</t>
+        </is>
+      </c>
       <c r="M113" s="30">
         <f>IF(ISNUMBER(SEARCH("/dp/",L113)),MID(L113,SEARCH("/dp/",L113)+4,10),"")</f>
         <v/>
       </c>
-      <c r="N113" s="28" t="n"/>
-      <c r="O113" s="29" t="n"/>
+      <c r="N113" s="28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B00JJVBXHK?tag=beastlyfacts-20</t>
+        </is>
+      </c>
+      <c r="O113" s="29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="P113" s="31" t="n"/>
-      <c r="Q113" s="29" t="n"/>
-      <c r="R113" s="32" t="n"/>
-      <c r="S113" s="28" t="n"/>
+      <c r="Q113" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R113" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="S113" s="28" t="inlineStr">
+        <is>
+          <t>PHOTO NEEDED: product-343.jpg = Josh's Frogs LECA Expanded Clay Pebbles (amazon.com/dp/B00JJVBXHK); product-344.jpg = Josh's Frogs Terrarium Substrate Barrier, 24x18 in (amazon.com/dp/B07D2KLX43)
+Catalog slug: leca-joshs-frogs-false-bottom, substrate-barrier-joshs-frogs-24x18. Also added: Josh's Frogs Terrarium Substrate Barrier, 24x18 in (https://www.amazon.com/dp/B07D2KLX43).</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="45" t="inlineStr">

</xml_diff>